<commit_message>
Update reviewed weekly content through September 27
</commit_message>
<xml_diff>
--- a/.batch-rewrite/weekly-content-ja-kr-2026-09-21.xlsx
+++ b/.batch-rewrite/weekly-content-ja-kr-2026-09-21.xlsx
@@ -1294,7 +1294,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>おはようございます。九月二十二日、火曜日の朝です。[PAUSE]駐輪場を通りかかると、誰かの自転車のかごに、コスモスが一輪、そっと挿してありました。庭から摘んできたのでしょうか、持ち主への小さな贈り物のように見えました。花を挿した人の姿は見当たりませんでしたが、朝の空気が少しだけ華やいだ気がします。近くに立っていた自転車には、まだ夏の名残のひまわりのシールが貼られていて、季節の変わり目をそっと教えてくれるようでした。[PAUSE]実は今日九月二十二日は、カレンダーの上では「休日」にあたる日です。昨日の敬老の日と、明日の秋分の日、その両方に祝日が重なっているため、法律の定めでその間の一日も休日になるのだそうです。今年は土曜日から数えて五連休となる、いわゆるシルバーウィークの真ん中にあたります。昨日、敬老の日を迎えられた皆様に、あらためて心からのお祝いを申し上げます。[PAUSE]彼岸の入りを過ぎ、朝の空気にひんやりとした感触が混じるようになりました。日中との気温差が大きくなる頃ですので、脱ぎ着しやすい一枚を鞄に入れておくと安心です。お墓参りや仏壇のお供えを準備される方も、この時期は多いかもしれませんね。[PAUSE]見返りを求めない小さな贈り物ほど、受け取った側の心に長く残るものかもしれません。花を挿した人は、きっと今日もいつも通りの一日を過ごしているだけなのでしょう。それでも、その何気ない行いが、見知らぬ誰かの朝を少し明るくしていました。[PAUSE]今日も、どなたかの一日に、そんな小さな彩りがありますように。良い一日をお過ごしください。[PAUSE]それでは、こもれび便りをまた明日も。</t>
+          <t>おはようございます。九月二十二日、火曜日の朝です。[PAUSE]駐輪場を通りかかると、誰かの自転車のかごに、コスモスが一輪、そっと挿してありました。庭から摘んできたのでしょうか、持ち主への小さな贈り物のように見えました。花を挿した人の姿は見当たりませんでしたが、朝の空気が少しだけ華やいだ気がします。近くに立っていた自転車には、まだ夏の名残のひまわりのシールが貼られていて、季節の変わり目をそっと教えてくれるようでした。[PAUSE]実は今日九月二十二日は、カレンダーの上では「休日」にあたる日です。昨日の敬老の日と明日の秋分の日に挟まれているため、祝日法の定めにより、その間の今日も休日になります。今年は土曜日から五日間続く、いわゆるシルバーウィークの真ん中にあたります。暦の並びによって生まれた、少し珍しい秋の休日です。昨日、敬老の日を迎えられた皆様に、あらためて心からのお祝いを申し上げます。[PAUSE]彼岸の入りを過ぎ、朝の空気にひんやりとした感触が混じるようになりました。日中との気温差が大きくなる頃ですので、脱ぎ着しやすい一枚を鞄に入れておくと安心です。お墓参りや仏壇のお供えを準備される方も、この時期は多いかもしれませんね。[PAUSE]見返りを求めない小さな贈り物ほど、受け取った側の心に長く残るものかもしれません。花を挿した人は、きっと今日もいつも通りの一日を過ごしているだけなのでしょう。それでも、その何気ない行いが、見知らぬ誰かの朝を少し明るくしていました。[PAUSE]今日も、どなたかの一日に、そんな小さな彩りがありますように。良い一日をお過ごしください。[PAUSE]それでは、こもれび便りをまた明日も。</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>こんにちは。お昼の脳トレクイズの時間です。今日は、頭の中だけで計算する、やさしい暗算の問題を五つご用意しました。紙とペンは使わずに、ゆっくり考えてみてくださいね。焦らなくて大丈夫です、自分のペースで進めましょう。指を使っても、声に出して数えても構いません、答えにたどり着くまでの過程を楽しんでいただければと思います。[PAUSE]最初の問題です。十七足す二十六は、いくつになるでしょうか。[PAUSE]正解は四十三です。十七を二十に近づけて、二十足す二十六は四十六、そこから足りない三を引くと四十三、というように考えると、暗算がぐっと楽になります。大きな数を割り出しやすい区切りの良い数に置き換えるというこの方法は、買い物の合計金額を頭の中でざっと見積もるときにも役立ちます。慣れてくると、レジに並んでいる間に自然と答えが浮かぶようになるかもしれません。[PAUSE]二問目です。八かける七は、いくつでしょうか。[PAUSE]正解は五十六です。九九の中でも、七の段は少し間違えやすいと言われていますが、八の段から考えると意外とすんなり出てくることもあります。学校で九九を覚えたときの、あの独特のリズムを思い出す方もいらっしゃるかもしれませんね。[PAUSE]三問目です。百から三十四を引くと、いくつになるでしょうか。[PAUSE]正解は六十六です。百からの引き算は、まず一の位から借りてくると考えるより、三十四を三十と四に分けて、百引く三十は七十、そこから四を引いて六十六、と段階を踏むと分かりやすくなります。きりの良い数から少しずつ引いていく方法は、暗算に慣れていない方ほど有効だと言われています。一度にすべてを計算しようとせず、二段階に分けるだけで、頭の中の負担がぐっと軽くなるものです。[PAUSE]四問目です。四十五足す三十八は、いくつでしょうか。[PAUSE]正解は八十三です。三十八を四十に近づけて、四十五足す四十は八十五、そこから多く足した二を引くと八十三になります。この「近い数に丸めてあとで調整する」というやり方は、どんな足し算にも応用できる便利な考え方で、大きな数になるほど威力を発揮します。[PAUSE]最後の問題です。六かける九は、いくつでしょうか。[PAUSE]正解は五十四です。九九の中でも六の段と九の段が重なるこの問題は、意外と忘れやすいと言われていますので、覚えておくと役立つかもしれません。九の段は、答えの十の位と一の位を足すと必ず九になるという面白い性質もあり、九一が九、九二十八というように順に確かめてみると、その規則性に気づく方も多いようです。[PAUSE]五問とも、いかがでしたでしょうか。今日も最後までお付き合いいただき、ありがとうございました。暗算は、毎日少しずつ続けることで、確実に鍛えられる力だと言われています。買い物のお釣りを計算するときなど、日常の中で試してみるのも良い練習になりますよ。指を使わずに答えが浮かんだときの、あのちょっとした達成感も、脳トレの醍醐味かもしれません。焦らず、ご自分のペースで続けていただければと思います。それでは、また明日のクイズでお会いしましょう。</t>
+          <t>こんにちは。お昼の脳トレクイズの時間です。今日は、頭の中だけで計算する、やさしい暗算の問題を五つご用意しました。紙とペンは使わずに、ゆっくり考えてみてくださいね。焦らなくて大丈夫です、自分のペースで進めましょう。指を使っても、声に出して数えても構いません、答えにたどり着くまでの過程を楽しんでいただければと思います。[PAUSE]最初の問題です。十七足す二十六は、いくつになるでしょうか。[PAUSE]正解は四十三です。十七を二十に近づけて、二十足す二十六は四十六、そこから足りない三を引くと四十三、というように考えると、暗算がぐっと楽になります。大きな数を割り出しやすい区切りの良い数に置き換えるというこの方法は、買い物の合計金額を頭の中でざっと見積もるときにも役立ちます。慣れてくると、レジに並んでいる間に自然と答えが浮かぶようになるかもしれません。[PAUSE]二問目です。八かける七は、いくつでしょうか。[PAUSE]正解は五十六です。九九の中でも、七の段は少し間違えやすいと言われていますが、八の段から考えると意外とすんなり出てくることもあります。学校で九九を覚えたときの、あの独特のリズムを思い出す方もいらっしゃるかもしれませんね。[PAUSE]三問目です。百から三十四を引くと、いくつになるでしょうか。[PAUSE]正解は六十六です。百からの引き算は、まず一の位から借りてくると考えるより、三十四を三十と四に分けて、百引く三十は七十、そこから四を引いて六十六、と段階を踏むと分かりやすくなります。きりの良い数から少しずつ引いていく方法は、暗算に慣れていない方ほど有効だと言われています。一度にすべてを計算しようとせず、二段階に分けるだけで、頭の中の負担がぐっと軽くなるものです。[PAUSE]四問目です。四十五足す三十八は、いくつでしょうか。[PAUSE]正解は八十三です。三十八を四十に近づけて、四十五足す四十は八十五、そこから多く足した二を引くと八十三になります。この「近い数に丸めてあとで調整する」というやり方は、どんな足し算にも応用できる便利な考え方で、大きな数になるほど威力を発揮します。[PAUSE]最後の問題です。六かける九は、いくつでしょうか。[PAUSE]正解は五十四です。九九の中でも六の段と九の段が重なるこの問題は、意外と忘れやすいと言われていますので、覚えておくと役立つかもしれません。九の段は、答えの十の位と一の位を足すと必ず九になるという面白い性質もあり、九一が九、九二が十八というように順に確かめてみると、その規則性に気づく方も多いようです。[PAUSE]五問とも、いかがでしたでしょうか。今日も最後までお付き合いいただき、ありがとうございました。暗算は、毎日少しずつ続けることで、確実に鍛えられる力だと言われています。買い物のお釣りを計算するときなど、日常の中で試してみるのも良い練習になりますよ。指を使わずに答えが浮かんだときの、あのちょっとした達成感も、脳トレの醍醐味かもしれません。焦らず、ご自分のペースで続けていただければと思います。それでは、また明日のクイズでお会いしましょう。</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>夜九時になると、隣の空き部屋にだけ、いつも決まって静かに明かりが灯ります。住んでいるはずのない部屋の窓に、なぜ光が見えるのか、多恵子さんはしばらくの間、不思議に思っていました。[PAUSE]こんばんは。今夜も、こもれび便りに、しばらくお付き合いください。[PAUSE]多恵子さんの隣家は、半年前に一人暮らしのご主人を亡くされた家でした。息子さん夫婦は遠方に住んでおり、家は今、誰も住んでいないはずでした。それなのに、毎晩九時になると決まって二階の窓に明かりが灯るのです。最初は空き巣か何かかと不安になりましたが、翌朝早くに明かりが消えていることに気づき、どうも少し様子が違うと感じるようになりました。[PAUSE]ある晩、思い切って様子を見に行くと、庭先に息子さんの姿がありました。聞けば、仕事帰りに毎晩立ち寄り、タイマー式の照明をつけてから帰っているのだそうです。「空き家だと分かると、近所に迷惑がかかるかもしれないので」とも言っていましたが、多恵子さんには、それだけが理由ではないように見えました。[PAUSE]「父が生きていた頃、いつも九時になると、この部屋の灯りで居間を照らしていたんです。灯りが消えたままだと、なんだかまだ父がいなくなったことを、認めきれない気がして」。息子さんは、少し照れくさそうにそう打ち明けてくれました。仕事で疲れていても、この習慣だけは欠かしたことがないのだといいます。多恵子さんは、その言葉に胸を打たれました。[PAUSE]それから、多恵子さんも自然と、夜九時にふと窓の外を見るのが、小さな習慣になりました。今日も変わらず明かりが灯っている。それを確かめるだけで、誰かがこの家を大切に思い続けているのだと感じられて、不思議と安心するのだそうです。息子さんとも、それをきっかけに顔を合わせれば挨拶を交わす仲になりました。[PAUSE]人という存在は、目に見える形がなくなっても、誰かの心の中で、明かりを灯し続けることができるのかもしれません。悲しみというものを急いで片付けなくても、こうして小さな習慣の中で、少しずつ受け止めていく時間もあるのですね。今夜も、大切な人を想う灯りが、どこかで静かに揺れていますように。今夜もここまでお付き合いいただき、本当にありがとうございました。</t>
+          <t>夜九時になると、誰も住んでいないはずの隣家の二階に、決まって明かりが灯ります。その理由を知った夜、多恵子さんは、自分もまた長いあいだ消せずにいた心の灯りに気づきました。[PAUSE]こんばんは。今夜も、こもれび便りに、しばらくお付き合いください。[PAUSE]多恵子さんの隣家では、半年前まで一人暮らしの正雄さんが暮らしていました。朝に顔を合わせれば天気の話をし、庭で採れた柿を分け合うような、近すぎず遠すぎない隣人でした。正雄さんが亡くなり、遠方に住む息子夫婦が家を片づけてからは、雨戸も閉じられ、庭の鉢植えだけが季節に取り残されたように並んでいました。[PAUSE]それなのに、毎晩九時になると二階の窓に柔らかな光が灯り、十一時には消えるのです。最初の数日は、息子さんが片づけに来ているのだろうと思いました。しかし、人影も車も見えない夜が続き、多恵子さんは空き巣や漏電ではないかと心配になりました。町内会へ知らせる前に一度確かめようと、ある夕方、庭先を見に行きました。[PAUSE]門の前で会ったのは、正雄さんの息子の直人さんでした。直人さんは週に一度だけ家を訪れ、二階の照明が毎晩九時から二時間点くようタイマーを確かめ、郵便物や庭の様子を見ているのだと説明しました。「空き家だと分からないようにするためです」と笑いましたが、その声は少しだけ寂しそうでした。[PAUSE]多恵子さんが黙って待っていると、直人さんはゆっくり話し始めました。正雄さんは生前、夜九時になると二階の机で日記を書いていました。仕事で帰りが遅かった直人さんは、駅から見えるその窓の灯りを確認すると、父が元気でいると安心できたそうです。「亡くなったあと、真っ暗な窓を見るのがつらくて。まだ父がいない家に慣れないんです」。[PAUSE]多恵子さんは、その言葉を聞いて、自分の夫を亡くした頃を思い出しました。食卓から夫の湯飲みを片づけられず、半年ほど毎朝二つのお茶を淹れていたことがあります。周囲には早く気持ちを切り替えるよう励まされましたが、その湯飲みを一つにするまでには、自分にしか分からない時間が必要でした。[PAUSE]「無理に消さなくてもいいんじゃないかしら」。多恵子さんがそう言うと、直人さんは驚いたように顔を上げました。「私も、夫の湯飲みを長いこと片づけられなかったの。でも、ある朝、一つだけ淹れても寂しくない日が来たのよ。急がなくても、その日はちゃんと来るから」。直人さんはしばらく窓を見上げ、それから小さく頭を下げました。[PAUSE]それ以来、直人さんが家を見に来る土曜日には、多恵子さんも庭の掃除を少し手伝うようになりました。二人は正雄さんが育てていた鉢植えの名前を確かめ、枯れた枝を切り、新しい土を入れました。多恵子さんは正雄さんの好きだった柿の木のことを話し、直人さんは父が若い頃に書いた日記の一節を聞かせてくれました。悲しみについて正面から話さなくても、手を動かしているあいだ、二人の沈黙は不思議と重くありませんでした。[PAUSE]冬の初め、直人さんは多恵子さんに相談しました。家を売ることが決まり、翌月には照明も外すことになったというのです。「最後の日だけ、一緒に灯りを見てもらえませんか」。その夜、二人は多恵子さんの縁側に並び、九時に灯る窓を眺めました。直人さんは泣くことも言葉を飾ることもなく、ただ「父さん、今までありがとう」とつぶやきました。[PAUSE]十一時、灯りが静かに消えました。けれど直人さんの表情は、以前より穏やかでした。翌週、空になった隣家の窓辺には、正雄さんの鉢植えから分けた小さな椿が一鉢だけ残されていました。「多恵子さんに見てもらえたら、父も安心すると思います」と書かれた札が添えられていました。[PAUSE]春になると、その椿は赤い花を一つ咲かせました。多恵子さんは写真を撮り、直人さんへ送りました。ほどなく届いた返事には、「父の家の灯りは消えましたが、別の場所でまだ続いている気がします」とありました。[PAUSE]大切な人を失った悲しみには、誰かが決めた期限はありません。消せない灯りを無理に消すのではなく、そばで見守りながら、いつか別の形へ移していく。その時間に静かに寄り添うことも、人と人が支え合う一つの方法なのでしょう。今夜も、あなたの心に残る大切な灯りが、穏やかに揺れていますように。ここまでお付き合いいただき、ありがとうございました。</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>안녕하세요. 9월 22일 화요일 아침입니다.[PAUSE]오늘 아침 우유 배달을 오신 아저씨가 평소보다 한 톤 높은 목소리로 인사를 건네셨습니다. 무슨 좋은 일이 있으시냐고 여쭤보니, 딸이 오늘 첫 출근을 한다며 새벽부터 도시락을 싸 주고 나오는 길이라고 겸연쩍게 웃으셨습니다. 늘 무뚝뚝하게 우유병만 놓고 가시던 분이라, 그 들뜬 표정이 유독 눈에 오래 남았습니다.[PAUSE]오늘 9월 22일은 자동차 없는 날로 알려져 있습니다. 세계 여러 도시가 하루만이라도 자동차 대신 걷거나 자전거로 이동해 보자는 취지로 함께하는 날인데, 서울을 비롯한 여러 지자체에서도 매년 이 시기에 관련 캠페인을 벌이고 있습니다. 오늘 하루만큼은 가까운 거리를 걸어서 다녀 보는 것도 좋겠습니다.[PAUSE]추분을 하루 앞두고, 아침 공기에 제법 서늘한 기운이 섞여 듭니다. 낮과 밤의 기온 차가 커지는 시기이니, 가볍게 걸칠 겉옷 하나를 가방에 넣어 두시면 든든하겠습니다. 이맘때는 감기 기운도 슬쩍 찾아오기 쉬우니 따뜻한 차 한 잔도 챙겨 보시길 권해 드립니다.[PAUSE]누군가의 인생에서 처음이라는 순간은, 그 사람 곁의 다른 이들에게도 은근히 마음을 설레게 하는 힘이 있는 것 같습니다. 우유 아저씨의 딸은 오늘 하루 얼마나 긴장했을지, 얼마나 뿌듯했을지, 얼굴도 모르는 그 청년의 하루를 괜히 응원하게 되는 아침이었습니다.[PAUSE]오늘도 누군가의 하루에 그런 작은 설렘이 함께하길 바랍니다. 그럼 햇살 편지는 내일도 함께하겠습니다.</t>
+          <t>안녕하세요. 9월 22일 화요일 아침입니다.[PAUSE]오늘 아침 우유 배달을 오신 아저씨가 평소보다 한 톤 높은 목소리로 인사를 건네셨습니다. 무슨 좋은 일이 있으시냐고 여쭤보니, 딸이 오늘 첫 출근을 한다며 새벽부터 도시락을 싸 주고 나오는 길이라고 겸연쩍게 웃으셨습니다. 늘 무뚝뚝하게 우유병만 놓고 가시던 분이라, 그 들뜬 표정이 유독 눈에 오래 남았습니다.[PAUSE]오늘 9월 22일은 자동차 없는 날로 알려져 있습니다. 세계 여러 도시가 하루만이라도 자동차 대신 걷거나 자전거로 이동해 보자는 취지로 함께하는 날인데, 서울을 비롯한 여러 지자체에서도 매년 이 시기에 관련 캠페인을 벌이고 있습니다. 오늘 하루만큼은 가까운 거리를 걸어서 다녀 보는 것도 좋겠습니다.[PAUSE]추분을 하루 앞두고, 아침 공기에 제법 서늘한 기운이 섞여 듭니다. 낮과 밤의 기온 차가 커지는 시기이니, 가볍게 걸칠 겉옷 하나를 가방에 넣어 두시면 든든하겠습니다. 이맘때는 감기 기운도 슬쩍 찾아오기 쉬우니 따뜻한 차 한 잔도 챙겨 보시길 권해 드립니다.[PAUSE]누군가의 인생에서 처음이라는 순간은, 그 사람 곁의 다른 이들에게도 은근히 마음을 설레게 하는 힘이 있는 것 같습니다. 우유 아저씨의 딸은 오늘 하루 얼마나 긴장했을지, 얼마나 뿌듯했을지, 얼굴도 모르는 그 딸의 첫날을 괜히 응원하게 되는 아침이었습니다.[PAUSE]오늘도 누군가의 하루에 그런 작은 설렘이 함께하길 바랍니다. 그럼 햇살 편지는 내일도 함께하겠습니다.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>매일 오후 두 시가 되면, 경로당 구석 자리에는 늘 같은 분이 조용히 앉아 계셨습니다. 말없이 창밖만 바라보시던 그 자리의 의미를, 정숙 씨는 최근에야 알게 되었습니다.[PAUSE]안녕하세요. 오늘 밤도 햇살 편지와 함께 잠시 마음을 나누어 보시죠.[PAUSE]정숙 씨가 경로당 총무를 맡은 지 얼마 되지 않았을 때, 구석 자리에 앉아 화투도 치지 않고, 대화에도 잘 끼지 않는 어르신 한 분이 눈에 띄었습니다. 이름은 복순 할머니로, 몇 해 전 할아버지를 먼저 보내시고 혼자 지내고 계신 분이었습니다. 정숙 씨는 처음에는 그저 낯을 가리시나 보다 생각하고, 크게 신경 쓰지 않았습니다.[PAUSE]그러던 어느 날, 정숙 씨가 우연히 여쭤보니, 복순 할머니는 그 자리가 예전에 할아버지가 늘 앉으시던 자리였다고 말씀하셨습니다. 할아버지가 살아 계실 때는, 이 시간이면 늘 나란히 앉아 창밖 풍경을 바라보며 이런저런 이야기를 나누셨다는 것이었습니다. 지금은 말동무는 없지만, 그 시간, 그 자리에 앉아 있는 것만으로도 마음이 놓인다고 하셨습니다.[PAUSE]정숙 씨는 그 이야기를 듣고 나서, 오후 두 시가 되면 잠깐씩 복순 할머니 곁에 앉아, 굳이 대화를 강요하지 않고 그저 함께 창밖을 바라보는 시간을 갖기 시작했습니다. 처음에는 어색한 침묵이 흘렀지만, 며칠이 지나자 복순 할머니께서 먼저 옛날이야기를 꺼내 주시기 시작했습니다.[PAUSE]말을 많이 하지 않아도, 그저 곁에 있어 주는 것만으로 전해지는 마음이 있다는 것을, 정숙 씨는 그렇게 배워 갔습니다. 요즘은 다른 어르신들도 하나둘 그 자리 주변에 자연스럽게 모이게 되었고, 복순 할머니의 구석 자리는 이제 경로당에서 가장 따뜻한 이야기가 오가는 곳이 되었습니다.[PAUSE]누군가의 곁을 지킨다는 것은, 거창한 말이 아니라 그저 같은 시간, 같은 자리에 머무르는 것만으로도 충분할 때가 있는 것 같습니다. 오늘 밤도, 여러분 곁의 소중한 사람과 조용히 함께하는 시간을 가져 보시길 바랍니다. 여기까지 함께해 주셔서 감사합니다.</t>
+          <t>매일 오후 두 시가 되면, 경로당 구석 자리에는 늘 같은 분이 조용히 앉아 계셨습니다. 아무도 앉지 않은 옆 의자를 비워 둔 채 창밖만 바라보던 이유를, 정숙 씨는 한참 뒤에야 알게 되었습니다.[PAUSE]안녕하세요. 오늘 밤도 햇살 편지와 함께 잠시 마음을 나누어 보시죠.[PAUSE]정숙 씨가 경로당 총무를 맡은 지 얼마 되지 않았을 때였습니다. 오후 두 시만 되면 복순 할머니가 창가 구석에 앉았습니다. 다른 어르신들이 화투를 치거나 노래를 부를 때도, 복순 할머니는 대화에 끼지 않고 찻잔 두 개를 앞에 놓은 채 바깥 놀이터만 바라보았습니다. 한 잔은 천천히 비워졌지만, 맞은편 잔은 늘 그대로 식어 갔습니다.[PAUSE]몇몇 분은 자리를 두 개나 차지한다며 불편한 기색을 보이기도 했습니다. 정숙 씨도 처음에는 사람이 많을 때만이라도 찻잔을 치워 달라고 말씀드릴 생각이었습니다. 하지만 복순 할머니가 빈 의자 손잡이를 닦고, 비뚤어진 방석을 반듯하게 놓는 모습을 보고는 차마 말을 꺼내지 못했습니다.[PAUSE]비가 내리던 어느 날, 경로당에 사람이 거의 오지 않았습니다. 정숙 씨가 따뜻한 보리차를 건네며 조심스럽게 이유를 묻자, 복순 할머니는 한동안 찻잔만 바라보다가 입을 열었습니다. 그 자리는 삼 년 전 먼저 세상을 떠난 남편이 늘 앉던 자리였습니다. 두 사람은 장사를 마친 뒤 매일 오후 두 시에 경로당에 와서, 창밖을 보며 그날 있었던 일을 나누곤 했습니다.[PAUSE]“집에서는 혼자라는 생각만 드는데, 여기에 앉으면 이 사람이 잠깐 늦는 것 같아요.” 복순 할머니는 빈 의자를 가리키며 웃었습니다. 그 웃음이 애써 만든 것처럼 보여, 정숙 씨는 위로의 말을 서둘러 꺼내지 않았습니다. 그저 옆자리에 앉아 빗물이 창문을 타고 흐르는 모습을 함께 바라보았습니다.[PAUSE]그날부터 정숙 씨는 오후 두 시가 되면 십 분쯤 복순 할머니 곁에 앉았습니다. 어떤 날은 날씨 이야기를 했고, 어떤 날은 아무 말도 하지 않았습니다. 복순 할머니가 남편과 시장에서 국밥집을 운영했던 이야기, 새벽마다 함께 재료를 사러 다녔던 이야기, 마지막 병원에서 미처 고맙다는 말을 하지 못한 이야기를 먼저 꺼낼 때에만 조용히 귀를 기울였습니다.[PAUSE]몇 주 뒤, 복순 할머니가 경로당에 오지 않았습니다. 다음 날에도 구석 자리는 비어 있었습니다. 정숙 씨는 걱정이 되어 전화를 걸었지만 받지 않았고, 연락처에 적힌 딸에게 확인한 뒤 반찬 몇 가지를 챙겨 집을 찾아갔습니다. 복순 할머니는 감기로 몸살을 앓아 누워 있었습니다. 정숙 씨는 방을 정리하거나 잔소리를 하지 않고, 따뜻한 죽을 데워 식탁에 놓은 뒤 잠시 곁에 앉아 있었습니다.[PAUSE]“내가 경로당에 안 가니, 그 사람 자리도 혼자였겠네.” 복순 할머니가 힘없이 말하자 정숙 씨는 대답했습니다. “자리는 기다릴 수 있어요. 할머니부터 천천히 나으세요. 그리고 이제 그 자리에는 할머니를 기다리는 사람도 있어요.” 그 말을 들은 복순 할머니는 이불 끝을 만지며 오랫동안 아무 말이 없었습니다.[PAUSE]사흘 뒤, 복순 할머니가 다시 경로당에 왔습니다. 두 개였던 찻잔은 여전히 두 개였지만, 이번에는 빈 의자 옆에 정숙 씨가 앉을 작은 방석이 하나 더 놓여 있었습니다. 복순 할머니는 보리차를 따르며 남편이 좋아했던 오래된 노래 이야기를 먼저 꺼냈습니다.[PAUSE]시간이 지나면서 다른 어르신들도 구석 자리 가까이에 자연스럽게 모이기 시작했습니다. 누군가는 먼저 떠난 아내 이야기를 했고, 누군가는 멀리 사는 자식 이야기를 했습니다. 서로 해결책을 내놓지는 않았습니다. 대신 말이 끝날 때까지 기다려 주고, 빈 찻잔에 물을 채워 주었습니다. 한때 가장 조용했던 구석 자리가 경로당에서 가장 오래 이야기가 머무는 자리가 되었습니다.[PAUSE]어느 봄날, 복순 할머니는 남편 몫으로 두던 찻잔 대신 작은 화분 하나를 가져왔습니다. “이제 이 사람도 여기서 꽃구경하면 되지.” 화분에는 노란 수선화가 피어 있었습니다. 빈 의자는 치우지 않았지만, 그날부터는 누구든 쉬어 갈 수 있는 자리가 되었습니다.[PAUSE]누군가의 곁을 지킨다는 것은 아픔을 대신 없애 주는 일이 아닐지도 모릅니다. 서둘러 잊으라고 말하지 않고, 같은 시간과 같은 자리에 조용히 머물러 주는 것. 그러다 그 사람이 스스로 다음 찻잔을 내어 놓을 때까지 기다려 주는 것. 오늘 밤, 여러분 곁의 소중한 사람에게 그런 따뜻한 자리가 되어 주시길 바랍니다. 여기까지 함께해 주셔서 감사합니다.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>지하철 유실물센터 선반 한쪽에는, 일곱 달 전 열차 좌석에서 발견된 회색 코트 한 벌이 놓여 있었습니다. 그 안주머니에서 나온 낡은 카세트테이프 하나에는, 내일이면 폐기 도장이 찍힐 예정이었습니다.[PAUSE]안녕하세요. 이 늦은 시각까지 햇살 편지를 찾아 주셔서 고맙습니다. 마음을 편히 내려놓으시고, 오늘 하루의 무게를 잠시 내려놓아 보세요.[PAUSE]정옥 씨는 올해 예순셋, 서울 지하철 삼호선 한 환승역의 유실물센터에서 마흔두 해째 일해 온 사람입니다. 하루에도 수십 개씩 밀려드는 우산과 지갑, 휴대전화와 안경 사이에서, 정옥 씨는 물건 하나하나에 얽힌 사람의 흔적을 읽어 내는 일에 평생을 바쳐 왔습니다. 지갑 속 영수증의 접힌 모서리, 우산 손잡이에 밴 담배 냄새, 안경다리에 남은 매니큐어 자국. 남들에게는 그저 잡동사니였지만, 정옥 씨에게는 저마다의 사연을 품은 작은 단서들이었습니다.[PAUSE]정옥 씨가 이 일을 시작한 것은 스물한 살 무렵, 지하철 공사에 갓 입사해 임시로 배치된 유실물 창구에서였습니다. 처음에는 그저 서류를 정리하고 물건에 번호표를 붙이는 단순한 업무라 여겼지만, 어느 날 한 할머니가 잃어버린 손주의 돌 반지를 찾아 눈물을 흘리는 모습을 본 뒤로 생각이 완전히 바뀌었습니다. 정옥 씨는 그날 이후, 물건을 찾아 주는 일이 곧 사람의 마음 한 조각을 되돌려 주는 일이라는 것을 마음 깊이 새기게 되었습니다.[PAUSE]정옥 씨의 기억에 유독 남아 있는 사연도 하나 있었습니다. 십여 년 전, 시력이 몹시 나쁜 한 할아버지가 낡은 성적표 한 장을 찾으러 왔습니다. 자식이 어릴 적 받아 온 초등학교 성적표라고만 했을 뿐, 언제 어디서 잃어버렸는지조차 기억하지 못했습니다. 정옥 씨는 보름 넘게 접수함을 뒤진 끝에, 우연히 다른 서류 사이에 끼어 있던 그 성적표를 찾아냈습니다. 할아버지는 그것을 품에 안고 한참을 서 있다가, 작게 중얼거렸습니다. "이제 얼마 안 남은 눈으로, 마지막으로 한 번만 더 보고 싶었어요." 정옥 씨는 그날부터, 아무리 하찮아 보이는 물건이라도 함부로 넘기지 않는 버릇이 생겼습니다.[PAUSE]정옥 씨가 이 일에 유독 마음을 쏟게 된 데에는, 자신의 젊은 시절 경험도 한몫했습니다. 스물다섯 살 때, 정옥 씨는 돌아가신 어머니가 남긴 유일한 사진을 이사 도중 잃어버린 적이 있었습니다. 이삿짐센터에도, 옛집 주인에게도 수소문해 보았지만 끝내 찾지 못했고, 그 사진은 지금까지도 정옥 씨의 마음 한구석에 아쉬움으로 남아 있었습니다. 정옥 씨는 그 경험 때문에, 누군가에게는 하찮아 보일 물건 하나가 다른 누군가에게는 평생 다시 구할 수 없는 것일 수 있다는 사실을 누구보다 잘 알고 있었습니다.[PAUSE]마흔 해가 넘는 세월 동안, 정옥 씨는 자신만의 작은 방법들을 하나씩 쌓아 왔습니다. 지갑을 찾으러 온 사람에게는 지갑 속 카드 순서를 먼저 물었고, 우산을 찾는 사람에게는 손잡이를 쥐는 손의 위치를 살폈습니다. 정확한 설명 없이 그저 "제 물건이 맞을 거예요"라고만 하는 사람에게는 절대 물건을 내어 주지 않는 것이 정옥 씨의 원칙이었습니다. 그런 작은 확인들이 쌓여, 정옥 씨는 이 좁은 창구 안에서 나름의 신망을 얻어 왔습니다.[PAUSE]정옥 씨의 정년퇴직은 이제 삼 주 앞으로 다가와 있었습니다. 요란한 송별회도, 특별한 기념패도 없이, 그저 정해진 날짜가 되면 조용히 사무실 열쇠를 반납하고 나가는 것이 전부였습니다. 정옥 씨는 그 사실이 서운하다기보다는, 마흔두 해 동안 스쳐 간 수많은 물건과 사람들의 얼굴을 마음속으로 하나씩 정리하는 시간으로 삼고 있었습니다.[PAUSE]얼마 전 정옥 씨는, 함께 야간 근무를 서던 후배 직원에게 넌지시 이런 말을 들은 적이 있었습니다. "정옥 씨는 물건만 봐도 주인 성격이 보인다면서요." 정옥 씨는 웃으며 고개를 저었습니다. "그런 게 아니라, 그냥 오래 들여다보는 것뿐이에요. 사람이든 물건이든, 눈을 오래 두면 저절로 보이는 것들이 있더라고요." 그 말은 정옥 씨가 마흔두 해 동안 스스로에게 되뇌어 온 말이기도 했습니다.[PAUSE]그러던 어느 날 오후, 정옥 씨는 곧 폐기될 예정인 물품 목록을 정리하다가 회색 코트 한 벌 앞에서 손을 멈추었습니다. 일곱 달 전 막차 시간대에 승객 신고로 접수된 코트였는데, 안주머니 깊숙한 곳에서 손바닥만 한 카세트테이프가 하나 나왔습니다. 테이프 케이스에는 색이 바랜 파란 색연필로, "정원에게"라는 세 글자가 삐뚤빼뚤 적혀 있었습니다.[PAUSE]유실물 관련 규정에 따르면, 소유자를 찾지 못한 물품은 접수일로부터 법정 보관 기간인 여섯 달이 지나면 소유권이 국가로 넘어가, 가치가 있는 물품은 공매 절차를, 낡은 의류처럼 가치가 낮은 품목은 자선단체 기증이나 재활용 절차를 밟게 되어 있었습니다. 이 코트는 이미 그 여섯 달을 넘긴 상태였고, 내일 오전이면 폐기 목록에 최종 도장이 찍힐 예정이었습니다. 정옥 씨는 그 작은 테이프를 손에 쥔 채, 좀처럼 서류함에 다시 집어넣지 못했습니다.[PAUSE]회색 코트 자체는 딱히 특별할 것 없는 물건이었습니다. 이십 년은 됨 직한 오래된 남성용 코트로, 소매 끝이 해지고 단추 하나가 떨어져 나가 있었습니다. 처음 접수했을 당시 정옥 씨는 그저 흔한 분실물 중 하나로만 여기고 선반 번호를 매겨 두었을 뿐, 안주머니 속 테이프를 발견한 것은 폐기 목록을 정리하던 그날이 처음이었습니다.[PAUSE]정옥 씨는 창고 구석, 오래전부터 방치되어 있던 폐기 대상 전자제품 상자를 뒤져 낡은 워크맨 하나를 찾아냈습니다. 몇 해 전 어느 대학생이 찾으러 오지 않아 폐기 대기 중이던 물건이었습니다. 다른 폐건전지 몇 개를 조합해 겨우 전원이 들어오는 것을 확인한 뒤, 정옥 씨는 퇴근 시간이 지난 텅 빈 사무실에 홀로 남아 테이프를 밀어 넣었습니다.[PAUSE]지지직거리는 잡음이 한참 이어지다가, 이내 한 여성의 나긋한 목소리가 흘러나왔습니다. "옛날 옛날, 달빛 아래 사는 여우 한 마리가 있었어요." 동화를 읽어 주는 목소리였습니다. 잠시 후 어린아이의 웃음소리가 끼어들며, 여성의 말을 서툴게 따라 하는 소리가 겹쳐 들렸습니다. "엄마, 여우가 진짜 달을 먹었어?" 정옥 씨는 그 자리에 선 채, 오래도록 그 목소리를 다시 되감아 들었습니다.[PAUSE]테이프 중간쯤, 여성의 목소리가 문득 이렇게 말했습니다. "오늘은 삼월 열이렛날이야, 정원아. 아빠가 밤 기차 몰고 오시면, 우리 이 이야기 또 들려드리자." 정옥 씨는 그 한 문장에서, 아버지가 야간 근무를 하는 기관사였을지도 모른다는 짐작을, 그리고 이 테이프가 어느 평범한 저녁, 엄마가 아이를 위해 손수 녹음한 잠자리 이야기였을 것이라는 짐작을 동시에 떠올렸습니다.[PAUSE]테이프 끝자락에는 짤막한 기계음과 함께, 케이스 뒷면에 희미하게 찍힌 도장 자국이 남아 있었습니다. "인성전자수리"라는 상호와, 지워져 가는 전화번호 앞자리 몇 개였습니다. 정옥 씨는 그 흐릿한 도장을, 사무실 형광등 아래 몇 번이고 눈을 가늘게 뜨고 들여다보았습니다.[PAUSE]다음 날 아침, 정옥 씨는 이 사연을 팀장인 박 팀장에게 조심스럽게 전했습니다. 박 팀장은 정옥 씨의 이야기를 다 듣기도 전에 손을 내저었습니다. "정옥 씨, 저도 마음은 알겠는데요. 지난번 결혼반지 건 기억나시죠? 그때도 개인적으로 알아보러 다니시다가 감사에서 지적받았잖아요. 이번엔 정옥 씨 명의로 경고까지 올라가 있는 상태예요." 박 팀장의 목소리에는 단호함이 배어 있었습니다.[PAUSE]박 팀장이 언급한 결혼반지 사건은, 반년 전 정옥 씨가 근무 시간 중에 반지 안쪽에 새겨진 이니셜만으로 예식장 여러 곳에 일일이 전화를 돌리다가, 정작 그날 처리해야 할 분실물 대장 마감을 늦추었던 일이었습니다. 결과적으로 반지 주인은 찾았지만, 본사 감사에서는 업무 태만으로 지적을 받았고, 정옥 씨의 인사 기록에는 구두 경고가 남아 있었습니다.[PAUSE]박 팀장은 이어 말했습니다. "보관 기한이 지난 물품 중에서도, 그 테이프처럼 누군가의 목소리나 개인적인 사연이 그대로 담긴 것들은 사생활 보호 차원에서 반드시 정해진 날짜에 파쇄해야 합니다. 이건 제 재량이 아니라 규정이에요. 정옥 씨가 퇴직을 앞두고 계신 것도 알지만, 마지막까지 문제를 만들지는 말아 주셨으면 합니다." 정옥 씨는 그 말을 들으며 아무 대꾸도 하지 못한 채 고개만 끄덕였습니다.[PAUSE]사무실로 돌아온 정옥 씨는 한참을 창구 의자에 앉아 있었습니다. 규정을 어기면 마흔두 해 동안 쌓아 온 신뢰가 마지막에 흠집이 날 수도 있었고, 어쩌면 얼마 남지 않은 퇴직금에도 영향이 있을 수 있었습니다. 정옥 씨는 자신에게 되물었습니다. 이제 와서 굳이 위험을 감수할 이유가 있을까. 남은 삼 주만 조용히 채우면, 마흔두 해의 경력에 아무런 흠집 없이 물러날 수 있었습니다.[PAUSE]하지만 그 작은 테이프 속 아이의 웃음소리가, 정옥 씨의 머릿속을 떠나지 않았습니다. 정옥 씨는 결국, 근무 시간이 아닌 자신의 개인 시간을 써서 딱 하루만 더 알아보기로 마음먹었습니다. 다행히 폐기 서류에 최종 서명을 넣는 것은 정옥 씨의 몫이었고, 정옥 씨는 서류 처리를 이틀 늦추는 것으로 스스로 시간을 벌었습니다.[PAUSE]정옥 씨는 퇴근 후, 낡은 전화번호부와 오래된 지역 상가 지도를 뒤져 "인성전자수리"라는 상호를 찾아 나섰습니다. 도장에 남은 주소를 어렵게 짜맞춰 찾아간 곳은, 이제는 편의점으로 바뀌어 있었습니다. 편의점 직원은 그런 가게가 있었는지조차 모른다고 했습니다. 정옥 씨는 어둑해진 골목에 서서, 첫 번째 단서가 이렇게 허무하게 끊기는 것에 잠시 맥이 풀렸습니다.[PAUSE]다음 날, 정옥 씨는 구청 도서관에 들러 지역 옛 상공인 명부를 뒤진 끝에, 인성전자수리를 운영했던 노인 한 분의 연락처를 겨우 찾아냈습니다. 여든을 훌쩍 넘긴 노인은 전화 너머로 한참 뜸을 들이다가, "그런 손님이 한둘이었어야지요"라며 힘없이 웃었습니다. 정옥 씨는 실망감을 누르며, 혹시 강정원이라는 이름을 기억하시는지 다시 여쭈었습니다.[PAUSE]노인은 잠시 침묵하더니, "강정원이라면, 그 동네 살던 아이 이름 같은데. 확실친 않아요"라며 어렴풋한 기억을 더듬어 냈습니다. 정옥 씨는 우선 전화번호 안내 서비스를 통해 같은 이름을 쓰는 사람을 찾아 몇 군데 전화를 걸어 보았습니다. 첫 번째 사람은 아예 다른 지역 출신이었고, 두 번째 사람은 전화를 받자마자 스팸이냐며 끊어 버렸습니다. 정옥 씨는 한숨을 삼키며, 결국 직접 찾아가 보는 수밖에 없겠다고 마음먹었습니다.[PAUSE]노인이 알려 준 옛 주소를 들고, 정옥 씨는 다음 날 오후 반차를 내어 그 동네를 찾아갔습니다. 낡은 다세대 주택 문을 두드리자, 중년 남성이 나와 정옥 씨의 이야기를 듣더니 고개를 저었습니다. "저희 집엔 그런 이름 쓰는 사람 없었는데요. 잘못 찾아오신 것 같습니다." 남자는 이름이 같은 사람이 이 동네에만도 여럿일 거라며, 문을 도로 닫았습니다.[PAUSE]정옥 씨는 낯선 골목에 홀로 서서, 자신이 괜한 헛수고를 하고 있는 것은 아닌지 스스로에게 물었습니다. 명예도, 상급자의 인정도 걸려 있지 않은 이 일에, 남은 며칠을 이렇게 써도 되는 것인지 확신이 서지 않았습니다. 그날 밤, 정옥 씨는 지친 마음을 달래려 테이프를 다시 한번 처음부터 끝까지 들었습니다. 그러다 이전에는 흘려들었던 한 대목을 다시 발견했습니다. 여성의 목소리가 아이에게 이렇게 말하고 있었습니다. "내일은 언덕 위 유치원 가는 날이지? 선생님한테 이 이야기도 들려드리자."[PAUSE]정옥 씨는 다시 인성전자수리 노인에게 전화를 걸어, 언덕 위에 있던 유치원을 기억하시는지 물었습니다. 노인은 이번에는 비교적 또렷하게 대답했습니다. "아, 그 동네 언덕 위 유치원이라면 기억나요. 그 근처에서 몇 해 전에 큰불이 났었지요. 집이 여러 채 탔던 걸로 기억하는데." 정옥 씨는 그 말을 듣는 순간, 등줄기가 서늘해지는 것을 느꼈습니다.[PAUSE]정옥 씨는 다음 날 구청 안전관리과를 찾아가, 오래된 화재 기록을 열람할 수 있는지 문의했습니다. 담당자는 번거로운 얼굴을 했지만, 정옥 씨가 사정을 짧게 설명하자 옛 신문 축쇄판 자료를 함께 찾아 주었습니다. 두 사람은 먼지 쌓인 마이크로필름을 한 장 한 장 넘기며, 언덕 위 유치원이라는 단어가 나올 때까지 눈이 시리도록 화면을 들여다보았습니다. 그렇게 찾아낸 기사에는, 언덕 위 유치원 인근 주택에서 화재가 발생해 한 가정이 큰 피해를 입었고, 어린 아들 하나가 이웃집에 맡겨져 있던 덕분에 무사했다는 짧은 단신이 실려 있었습니다.[PAUSE]기사에는 아이의 이름 대신 성만 실려 있었지만, 정옥 씨는 그 동네 초등학교 행정실에 전화를 걸어, 화재 시기와 비슷한 시절 전학 기록이 있는 학생 중에 강씨 성을 가진 아이가 있었는지 조심스럽게 물었습니다. 행정실 직원은 재학생과 졸업생의 개인정보는 알려 드릴 수 없다며 정중히 거절했지만, 옛 졸업생들의 소식을 따로 모아 관리하는 총동문회 사무실이 있다고 귀띔해 주었습니다.[PAUSE]정옥 씨는 곧바로 총동문회에 연락을 넣었습니다. 담당자 역시 개인 신상 정보까지는 알려 줄 수 없다고 선을 그었지만, 몇 해 전 동문 소식지에 이미 공개적으로 실렸던 내용이라며 한 가지 사실을 알려 주었습니다. 비슷한 시기에 다니던 졸업생 가운데 한 명이, 지금은 인근 초등학교에서 교사로 재직 중이라는 것이었습니다. 이름은 강정원, 그리고 근무지는 정옥 씨의 집에서 그리 멀지 않은 초등학교였습니다.[PAUSE]정옥 씨는 다음 날 저녁, 수업이 끝난 초등학교 교무실을 찾아갔습니다. 마흔 줄에 접어든 강정원 씨는 낯선 방문객을 경계하는 얼굴이었지만, 정옥 씨가 조심스레 꺼낸 "정원에게"라는 세 글자와, 삼월 열이렛날이라는 날짜, 그리고 언덕 위 유치원 이야기를 듣는 순간 표정이 완전히 굳어졌습니다. "그걸 어떻게, 어떻게 알고 계세요." 정원 씨의 목소리가 떨리고 있었습니다.[PAUSE]정옥 씨가 가방에서 조심스럽게 카세트테이프를 꺼내 건네자, 정원 씨는 그 자리에 얼어붙은 듯 한참을 움직이지 못했습니다. 떨리는 손으로 테이프를 받아 든 정원 씨는, 낮은 목소리로 이야기를 시작했습니다. "저희 어머니가 돌아가신 게, 제가 일곱 살 때였어요. 그날 집에 불이 나서, 사진 한 장 남지 않았습니다. 저는 마침 이웃집에 맡겨져 있어서 화를 피했고요."[PAUSE]정원 씨는 말을 이었습니다. "아버지가 야간 기관사로 일하셔서, 어머니는 아버지 없는 밤마다 저한테 이야기를 지어 녹음해 주셨어요. 이 테이프가 아마 그중 마지막으로 녹음된 걸 거예요. 어머니 목소리가 담긴 건 이것 하나뿐이었는데, 불이 난 뒤로는 다 사라진 줄로만 알고 살았습니다." 정옥 씨는 그 말을 들으며, 자신이 왜 그토록 이 작은 테이프를 놓지 못했는지 비로소 이해할 수 있었습니다.[PAUSE]정원 씨는 이어, 코트가 어떻게 자신의 손을 떠나게 되었는지도 짐작이 간다며 설명을 덧붙였습니다. 화재 이후 어린 정원 씨를 거두어 키워 준 이모가 몇 해 전 세상을 떠나면서, 유품을 정리하던 친척들이 이모의 오래된 옷가지들을 자선단체에 통째로 기증했는데, 그 코트가 바로 그중 하나였을 것이라고 했습니다. 코트 안주머니에 테이프가 들어 있는 줄은, 정원 씨 자신도 전혀 모르고 있었습니다.[PAUSE]정옥 씨는 조심스럽게 물었습니다. "이모님 유품인 줄 모르고 넘겨 드렸다니, 혹시 서운하게 들리시진 않으셨어요." 정원 씨는 고개를 저으며 나직이 웃었습니다. "아니요. 오히려 다행이에요. 이모가 마지막까지 이걸 소중히 걸어 두셨던 거잖아요. 잃어버렸다고 생각했던 게, 이렇게 돌아왔으니까요."[PAUSE]정원 씨는 잠시 창밖을 바라보다가, 다시 정옥 씨 쪽으로 몸을 돌렸습니다. "사실 저는 어머니 목소리가 어땠는지도 가물가물했어요. 사진 한 장 없으니까, 시간이 지날수록 얼굴도 목소리도 점점 흐려지더라고요. 그런데 아까 잠깐 튼 부분에서, 어머니가 제 이름을 부르는 그 억양이, 듣자마자 그냥 온몸에 소름이 돋았습니다. 이게 진짜 우리 엄마구나, 하고요." 정옥 씨는 그 말을 들으며 자신도 모르게 눈시울이 붉어지는 것을 느꼈습니다.[PAUSE]정원 씨는 테이프를 두 손으로 꼭 쥔 채 한동안 말을 잇지 못하다가, 문득 정옥 씨에게 물었습니다. "이걸 찾으시려고, 규정까지 어기면서 애쓰셨다고 들었어요. 저한테는 이게 세상 전부인 물건이지만, 정옥 씨한테는 그냥 낡은 카세트테이프 하나였을 텐데, 왜 그렇게까지 하셨어요." 정옥 씨는 잠시 생각하다가 담담히 대답했습니다. "저도 잘 모르겠어요. 그냥, 이걸 그대로 부숴 버리면 다시는 되돌릴 수 없다는 게, 마음에 걸려서요."[PAUSE]정옥 씨가 사무실로 돌아와 이 일을 박 팀장에게 보고하자, 박 팀장은 잠시 말이 없다가 짧게 한숨을 내쉬었습니다. "정옥 씨, 규정은 규정이니 경고 기록은 그대로 남을 겁니다. 그건 저도 어쩔 수 없어요." 정옥 씨는 담담하게 고개를 끄덕였습니다. "괜찮습니다. 저는 이제 곧 나갈 사람인걸요." 박 팀장은 그 말에 잠시 정옥 씨를 바라보다가, "수고하셨습니다"라는 말을 짧게 남기고 자리를 떴습니다.[PAUSE]정옥 씨의 정년퇴직일이 마침내 다가왔습니다. 특별한 행사도, 꽃다발도 없이, 정옥 씨는 여느 날과 다름없이 아침 일찍 출근해 마지막으로 창구에 앉았습니다. 그날따라 분실물 신고가 유난히 많았고, 정옥 씨는 우산 세 개와 지갑 하나, 그리고 아이의 장갑 한 짝을 각각의 주인에게 돌려주었습니다.[PAUSE]퇴근 시간이 되어 짐을 정리하던 정옥 씨는, 서랍 맨 아래 칸에서 그동안 미처 주인을 찾지 못했던 작은 물건들의 사진을 모아 둔 낡은 수첩을 발견했습니다. 단추 하나, 빛바랜 사진 한 장, 이름 모를 열쇠 하나. 정옥 씨는 그 수첩을 버리지 않고, 조용히 가방 안에 챙겨 넣었습니다.[PAUSE]정옥 씨는 사무실을 나서기 전, 텅 빈 유실물 선반을 한 번 더 둘러보았습니다. 마흔두 해 동안 이 선반을 거쳐 간 무수한 물건들, 그리고 그 물건들 뒤에 숨어 있던 사람들의 사연이 스쳐 지나갔습니다. 정옥 씨는 문득, 자신이 이 일에서 배운 것은 대단한 기술이나 요령이 아니라, 남들이 하찮게 여기고 지나칠 법한 작은 것에 오래 눈길을 두는 태도였다는 것을 깨달았습니다.[PAUSE]정옥 씨는 후배들에게 무언가를 가르치거나 물려줄 생각은 하지 않았습니다. 다만 나가는 길에, 선반 옆 게시판에 붙어 있던 낡은 안내문 한 줄을 손수 고쳐 적었을 뿐입니다. "폐기 전, 다시 한번 들여다보기." 그것은 후임자를 위한 지침이라기보다, 마흔두 해 동안 정옥 씨 자신이 스스로에게 다짐해 온 말을 마지막으로 남겨 두는 것에 더 가까웠습니다.[PAUSE]며칠 뒤, 정옥 씨의 집으로 작은 소포 하나가 도착했습니다. 발신인은 강정원 씨였습니다. 소포 안에는 그 카세트테이프를 복원해 만든 디지털 음원 파일이 담긴 손바닥만 한 저장 장치와, 짧은 편지 한 장이 들어 있었습니다. "덕분에 어머니 목소리를 다시 들을 수 있게 됐습니다. 이제 이 목소리는 저 혼자만의 것이 아니라, 언젠가 제 아이에게도 들려줄 수 있는 것이 되었습니다. 정옥 씨가 아니었다면, 이 목소리는 정말로 사라졌을 겁니다."[PAUSE]오늘 밤의 이야기는 여기서 마치겠습니다. 정옥 씨가 마흔두 해 동안 지켜 온 것은, 크고 화려한 무언가가 아니라 남들이 쉽게 버리고 지나칠 작은 물건 하나에 담긴 마음을 끝까지 놓지 않는 태도였습니다. 편안한 마음으로, 부디 오늘 밤도 푹 주무시길 바랍니다. 좋은 꿈 꾸시고, 안녕히 주무세요.</t>
+          <t>지하철 유실물센터 선반 한쪽에는, 일곱 달 전 열차 좌석에서 발견된 회색 코트 한 벌이 놓여 있었습니다. 그 안주머니에서 나온 낡은 카세트테이프 하나에는, 내일이면 폐기 도장이 찍힐 예정이었습니다.[PAUSE]안녕하세요. 이 늦은 시각까지 햇살 편지를 찾아 주셔서 고맙습니다. 마음을 편히 내려놓으시고, 오늘 하루의 무게를 잠시 내려놓아 보세요.[PAUSE]정옥 씨는 올해 예순셋, 서울 지하철 3호선 한 환승역의 유실물센터에서 마흔두 해째 일해 온 사람입니다. 하루에도 수십 개씩 밀려드는 우산과 지갑, 휴대전화와 안경 사이에서, 정옥 씨는 물건 하나하나에 얽힌 사람의 흔적을 읽어 내는 일에 평생을 바쳐 왔습니다. 지갑 속 영수증의 접힌 모서리, 우산 손잡이에 밴 담배 냄새, 안경다리에 남은 매니큐어 자국. 남들에게는 그저 잡동사니였지만, 정옥 씨에게는 저마다의 사연을 품은 작은 단서들이었습니다.[PAUSE]정옥 씨가 이 일을 시작한 것은 스물한 살 무렵, 지하철 공사에 갓 입사해 임시로 배치된 유실물 창구에서였습니다. 처음에는 그저 서류를 정리하고 물건에 번호표를 붙이는 단순한 업무라 여겼지만, 어느 날 한 할머니가 잃어버린 손주의 돌 반지를 찾아 눈물을 흘리는 모습을 본 뒤로 생각이 완전히 바뀌었습니다. 정옥 씨는 그날 이후, 물건을 찾아 주는 일이 곧 사람의 마음 한 조각을 되돌려 주는 일이라는 것을 마음 깊이 새기게 되었습니다.[PAUSE]정옥 씨의 기억에 유독 남아 있는 사연도 하나 있었습니다. 십여 년 전, 시력이 몹시 나쁜 한 할아버지가 낡은 성적표 한 장을 찾으러 왔습니다. 자식이 어릴 적 받아 온 초등학교 성적표라고만 했을 뿐, 언제 어디서 잃어버렸는지조차 기억하지 못했습니다. 정옥 씨는 보름 넘게 접수함을 뒤진 끝에, 우연히 다른 서류 사이에 끼어 있던 그 성적표를 찾아냈습니다. 할아버지는 그것을 품에 안고 한참을 서 있다가, 작게 중얼거렸습니다. "이제 얼마 안 남은 눈으로, 마지막으로 한 번만 더 보고 싶었어요." 정옥 씨는 그날부터, 아무리 하찮아 보이는 물건이라도 함부로 넘기지 않는 버릇이 생겼습니다.[PAUSE]정옥 씨가 이 일에 유독 마음을 쏟게 된 데에는, 자신의 젊은 시절 경험도 한몫했습니다. 스물다섯 살 때, 정옥 씨는 돌아가신 어머니가 남긴 유일한 사진을 이사 도중 잃어버린 적이 있었습니다. 이삿짐센터에도, 옛집 주인에게도 수소문해 보았지만 끝내 찾지 못했고, 그 사진은 지금까지도 정옥 씨의 마음 한구석에 아쉬움으로 남아 있었습니다. 정옥 씨는 그 경험 때문에, 누군가에게는 하찮아 보일 물건 하나가 다른 누군가에게는 평생 다시 구할 수 없는 것일 수 있다는 사실을 누구보다 잘 알고 있었습니다.[PAUSE]마흔 해가 넘는 세월 동안, 정옥 씨는 자신만의 작은 방법들을 하나씩 쌓아 왔습니다. 지갑을 찾으러 온 사람에게는 지갑 속 카드 순서를 먼저 물었고, 우산을 찾는 사람에게는 손잡이를 쥐는 손의 위치를 살폈습니다. 정확한 설명 없이 그저 "제 물건이 맞을 거예요"라고만 하는 사람에게는 절대 물건을 내어 주지 않는 것이 정옥 씨의 원칙이었습니다. 그런 작은 확인들이 쌓여, 정옥 씨는 이 좁은 창구 안에서 나름의 신망을 얻어 왔습니다.[PAUSE]정옥 씨의 정년퇴직은 이제 삼 주 앞으로 다가와 있었습니다. 요란한 송별회도, 특별한 기념패도 없이, 그저 정해진 날짜가 되면 조용히 사무실 열쇠를 반납하고 나가는 것이 전부였습니다. 정옥 씨는 그 사실이 서운하다기보다는, 마흔두 해 동안 스쳐 간 수많은 물건과 사람들의 얼굴을 마음속으로 하나씩 정리하는 시간으로 삼고 있었습니다.[PAUSE]얼마 전 정옥 씨는, 함께 야간 근무를 서던 후배 직원에게 넌지시 이런 말을 들은 적이 있었습니다. "정옥 씨는 물건만 봐도 주인 성격이 보인다면서요." 정옥 씨는 웃으며 고개를 저었습니다. "그런 게 아니라, 그냥 오래 들여다보는 것뿐이에요. 사람이든 물건이든, 눈을 오래 두면 저절로 보이는 것들이 있더라고요." 그 말은 정옥 씨가 마흔두 해 동안 스스로에게 되뇌어 온 말이기도 했습니다.[PAUSE]그러던 어느 날 오후, 정옥 씨는 곧 폐기될 예정인 물품 목록을 정리하다가 회색 코트 한 벌 앞에서 손을 멈추었습니다. 일곱 달 전 막차 시간대에 승객 신고로 접수된 코트였는데, 안주머니 깊숙한 곳에서 손바닥만 한 카세트테이프가 하나 나왔습니다. 테이프 케이스에는 색이 바랜 파란 색연필로, "정원에게"라는 세 글자가 삐뚤빼뚤 적혀 있었습니다.[PAUSE]유실물 관련 절차에 따르면, 소유자를 찾지 못한 물품은 법정 보관 기간인 여섯 달 동안 보관됩니다. 습득자가 소유권을 포기한 물품은 그 기간이 지난 뒤 관계 기관의 결정에 따라 국고 귀속이나 양여, 폐기 절차로 넘어갈 수 있었습니다. 이 코트는 이미 그 여섯 달을 넘긴 상태였고, 내일 오전이면 폐기 목록에 최종 도장이 찍힐 예정이었습니다. 정옥 씨는 그 작은 테이프를 손에 쥔 채, 좀처럼 서류함에 다시 집어넣지 못했습니다.[PAUSE]회색 코트 자체는 딱히 특별할 것 없는 물건이었습니다. 이십 년은 됨 직한 오래된 남성용 코트로, 소매 끝이 해지고 단추 하나가 떨어져 나가 있었습니다. 처음 접수했을 당시 정옥 씨는 그저 흔한 분실물 중 하나로만 여기고 선반 번호를 매겨 두었을 뿐, 안주머니 속 테이프를 발견한 것은 폐기 목록을 정리하던 그날이 처음이었습니다.[PAUSE]정옥 씨는 창고 구석, 오래전부터 방치되어 있던 폐기 대상 전자제품 상자를 뒤져 낡은 워크맨 하나를 찾아냈습니다. 몇 해 전 어느 대학생이 찾으러 오지 않아 폐기 대기 중이던 물건이었습니다. 다른 폐건전지 몇 개를 조합해 겨우 전원이 들어오는 것을 확인한 뒤, 정옥 씨는 퇴근 시간이 지난 텅 빈 사무실에 홀로 남아 테이프를 밀어 넣었습니다.[PAUSE]지지직거리는 잡음이 한참 이어지다가, 이내 한 여성의 나긋한 목소리가 흘러나왔습니다. "옛날 옛날, 달빛 아래 사는 여우 한 마리가 있었어요." 동화를 읽어 주는 목소리였습니다. 잠시 후 어린아이의 웃음소리가 끼어들며, 여성의 말을 서툴게 따라 하는 소리가 겹쳐 들렸습니다. "엄마, 여우가 진짜 달을 먹었어?" 정옥 씨는 그 자리에 선 채, 오래도록 그 목소리를 다시 되감아 들었습니다.[PAUSE]테이프 중간쯤, 여성의 목소리가 문득 이렇게 말했습니다. "오늘은 삼월 열이렛날이야, 정원아. 아빠가 밤 기차 몰고 오시면, 우리 이 이야기 또 들려드리자." 정옥 씨는 그 한 문장에서, 아버지가 야간 근무를 하는 기관사였을지도 모른다는 짐작을, 그리고 이 테이프가 어느 평범한 저녁, 엄마가 아이를 위해 손수 녹음한 잠자리 이야기였을 것이라는 짐작을 동시에 떠올렸습니다.[PAUSE]테이프 끝자락에는 짤막한 기계음과 함께, 케이스 뒷면에 희미하게 찍힌 도장 자국이 남아 있었습니다. "인성전자수리"라는 상호와, 지워져 가는 전화번호 앞자리 몇 개였습니다. 정옥 씨는 그 흐릿한 도장을, 사무실 형광등 아래 몇 번이고 눈을 가늘게 뜨고 들여다보았습니다.[PAUSE]다음 날 아침, 정옥 씨는 이 사연을 팀장인 박 팀장에게 조심스럽게 전했습니다. 박 팀장은 정옥 씨의 이야기를 다 듣기도 전에 손을 내저었습니다. "정옥 씨, 저도 마음은 알겠는데요. 지난번 결혼반지 건 기억나시죠? 그때도 개인적으로 알아보러 다니시다가 감사에서 지적받았잖아요. 이번엔 정옥 씨 명의로 경고까지 올라가 있는 상태예요." 박 팀장의 목소리에는 단호함이 배어 있었습니다.[PAUSE]박 팀장이 언급한 결혼반지 사건은, 반년 전 정옥 씨가 근무 시간 중에 반지 안쪽에 새겨진 이니셜만으로 예식장 여러 곳에 일일이 전화를 돌리다가, 정작 그날 처리해야 할 분실물 대장 마감을 늦추었던 일이었습니다. 결과적으로 반지 주인은 찾았지만, 본사 감사에서는 업무 태만으로 지적을 받았고, 정옥 씨의 인사 기록에는 구두 경고가 남아 있었습니다.[PAUSE]박 팀장은 이어 말했습니다. "보관 기한이 지난 물품 중에서도, 그 테이프처럼 누군가의 목소리나 개인적인 사연이 그대로 담긴 것들은 사생활 보호 차원에서 반드시 정해진 날짜에 파쇄해야 합니다. 이건 제 재량이 아니라 규정이에요. 정옥 씨가 퇴직을 앞두고 계신 것도 알지만, 마지막까지 문제를 만들지는 말아 주셨으면 합니다." 정옥 씨는 그 말을 들으며 아무 대꾸도 하지 못한 채 고개만 끄덕였습니다.[PAUSE]사무실로 돌아온 정옥 씨는 한참을 창구 의자에 앉아 있었습니다. 규정을 어기면 마흔두 해 동안 쌓아 온 신뢰가 마지막에 흠집이 날 수도 있었고, 어쩌면 얼마 남지 않은 퇴직금에도 영향이 있을 수 있었습니다. 정옥 씨는 자신에게 되물었습니다. 이제 와서 굳이 위험을 감수할 이유가 있을까. 남은 삼 주만 조용히 채우면, 마흔두 해의 경력에 아무런 흠집 없이 물러날 수 있었습니다.[PAUSE]하지만 그 작은 테이프 속 아이의 웃음소리가, 정옥 씨의 머릿속을 떠나지 않았습니다. 정옥 씨는 결국, 근무 시간이 아닌 자신의 개인 시간을 써서 딱 하루만 더 알아보기로 마음먹었습니다. 다행히 폐기 서류에 최종 서명을 넣는 것은 정옥 씨의 몫이었고, 정옥 씨는 서류 처리를 이틀 늦추는 것으로 스스로 시간을 벌었습니다.[PAUSE]정옥 씨는 퇴근 후, 낡은 전화번호부와 오래된 지역 상가 지도를 뒤져 "인성전자수리"라는 상호를 찾아 나섰습니다. 도장에 남은 주소를 어렵게 짜맞춰 찾아간 곳은, 이제는 편의점으로 바뀌어 있었습니다. 편의점 직원은 그런 가게가 있었는지조차 모른다고 했습니다. 정옥 씨는 어둑해진 골목에 서서, 첫 번째 단서가 이렇게 허무하게 끊기는 것에 잠시 맥이 풀렸습니다.[PAUSE]다음 날, 정옥 씨는 구청 도서관에 들러 지역 옛 상공인 명부를 뒤진 끝에, 인성전자수리를 운영했던 노인 한 분의 연락처를 겨우 찾아냈습니다. 여든을 훌쩍 넘긴 노인은 전화 너머로 한참 뜸을 들이다가, "그런 손님이 한둘이었어야지요"라며 힘없이 웃었습니다. 정옥 씨는 실망감을 누르며, 혹시 강정원이라는 이름을 기억하시는지 다시 여쭈었습니다.[PAUSE]노인은 잠시 침묵하더니, "강정원이라면, 그 동네 살던 아이 이름 같은데. 확실친 않아요"라며 어렴풋한 기억을 더듬어 냈습니다. 정옥 씨는 우선 전화번호 안내 서비스를 통해 같은 이름을 쓰는 사람을 찾아 몇 군데 전화를 걸어 보았습니다. 첫 번째 사람은 아예 다른 지역 출신이었고, 두 번째 사람은 전화를 받자마자 스팸이냐며 끊어 버렸습니다. 정옥 씨는 한숨을 삼키며, 결국 직접 찾아가 보는 수밖에 없겠다고 마음먹었습니다.[PAUSE]노인이 알려 준 옛 주소를 들고, 정옥 씨는 다음 날 오후 반차를 내어 그 동네를 찾아갔습니다. 낡은 다세대 주택 문을 두드리자, 중년 남성이 나와 정옥 씨의 이야기를 듣더니 고개를 저었습니다. "저희 집엔 그런 이름 쓰는 사람 없었는데요. 잘못 찾아오신 것 같습니다." 남자는 이름이 같은 사람이 이 동네에만도 여럿일 거라며, 문을 도로 닫았습니다.[PAUSE]정옥 씨는 낯선 골목에 홀로 서서, 자신이 괜한 헛수고를 하고 있는 것은 아닌지 스스로에게 물었습니다. 명예도, 상급자의 인정도 걸려 있지 않은 이 일에, 남은 며칠을 이렇게 써도 되는 것인지 확신이 서지 않았습니다. 그날 밤, 정옥 씨는 지친 마음을 달래려 테이프를 다시 한번 처음부터 끝까지 들었습니다. 그러다 이전에는 흘려들었던 한 대목을 다시 발견했습니다. 여성의 목소리가 아이에게 이렇게 말하고 있었습니다. "내일은 언덕 위 유치원 가는 날이지? 선생님한테 이 이야기도 들려드리자."[PAUSE]정옥 씨는 다시 인성전자수리 노인에게 전화를 걸어, 언덕 위에 있던 유치원을 기억하시는지 물었습니다. 노인은 이번에는 비교적 또렷하게 대답했습니다. "아, 그 동네 언덕 위 유치원이라면 기억나요. 그 근처에서 몇 해 전에 큰불이 났었지요. 집이 여러 채 탔던 걸로 기억하는데." 정옥 씨는 그 말을 듣는 순간, 등줄기가 서늘해지는 것을 느꼈습니다.[PAUSE]정옥 씨는 다음 날 구청 안전관리과를 찾아가, 오래된 화재 기록을 열람할 수 있는지 문의했습니다. 담당자는 번거로운 얼굴을 했지만, 정옥 씨가 사정을 짧게 설명하자 옛 신문 축쇄판 자료를 함께 찾아 주었습니다. 두 사람은 먼지 쌓인 마이크로필름을 한 장 한 장 넘기며, 언덕 위 유치원이라는 단어가 나올 때까지 눈이 시리도록 화면을 들여다보았습니다. 그렇게 찾아낸 기사에는, 언덕 위 유치원 인근 주택에서 화재가 발생해 한 가정이 큰 피해를 입었고, 어린 아들 하나가 이웃집에 맡겨져 있던 덕분에 무사했다는 짧은 단신이 실려 있었습니다.[PAUSE]기사에는 아이의 이름 대신 성만 실려 있었지만, 정옥 씨는 그 동네 초등학교 행정실에 전화를 걸어, 화재 시기와 비슷한 시절 전학 기록이 있는 학생 중에 강씨 성을 가진 아이가 있었는지 조심스럽게 물었습니다. 행정실 직원은 재학생과 졸업생의 개인정보는 알려 드릴 수 없다며 정중히 거절했지만, 옛 졸업생들의 소식을 따로 모아 관리하는 총동문회 사무실이 있다고 귀띔해 주었습니다.[PAUSE]정옥 씨는 곧바로 총동문회에 연락을 넣었습니다. 담당자 역시 개인 신상 정보까지는 알려 줄 수 없다고 선을 그었지만, 몇 해 전 동문 소식지에 이미 공개적으로 실렸던 내용이라며 한 가지 사실을 알려 주었습니다. 비슷한 시기에 다니던 졸업생 가운데 한 명이, 지금은 인근 초등학교에서 교사로 재직 중이라는 것이었습니다. 이름은 강정원, 그리고 근무지는 정옥 씨의 집에서 그리 멀지 않은 초등학교였습니다.[PAUSE]정옥 씨는 다음 날 저녁, 수업이 끝난 초등학교 교무실을 찾아갔습니다. 마흔 줄에 접어든 강정원 씨는 낯선 방문객을 경계하는 얼굴이었지만, 정옥 씨가 조심스레 꺼낸 "정원에게"라는 세 글자와, 삼월 열이렛날이라는 날짜, 그리고 언덕 위 유치원 이야기를 듣는 순간 표정이 완전히 굳어졌습니다. "그걸 어떻게, 어떻게 알고 계세요." 정원 씨의 목소리가 떨리고 있었습니다.[PAUSE]정옥 씨가 가방에서 조심스럽게 카세트테이프를 꺼내 건네자, 정원 씨는 그 자리에 얼어붙은 듯 한참을 움직이지 못했습니다. 떨리는 손으로 테이프를 받아 든 정원 씨는, 낮은 목소리로 이야기를 시작했습니다. "저희 어머니가 돌아가신 게, 제가 일곱 살 때였어요. 그날 집에 불이 나서, 사진 한 장 남지 않았습니다. 저는 마침 이웃집에 맡겨져 있어서 화를 피했고요."[PAUSE]정원 씨는 말을 이었습니다. "아버지가 야간 기관사로 일하셔서, 어머니는 아버지 없는 밤마다 저한테 이야기를 지어 녹음해 주셨어요. 이 테이프가 아마 그중 마지막으로 녹음된 걸 거예요. 어머니 목소리가 담긴 건 이것 하나뿐이었는데, 불이 난 뒤로는 다 사라진 줄로만 알고 살았습니다." 정옥 씨는 그 말을 들으며, 자신이 왜 그토록 이 작은 테이프를 놓지 못했는지 비로소 이해할 수 있었습니다.[PAUSE]정원 씨는 이어, 코트가 어떻게 자신의 손을 떠나게 되었는지도 짐작이 간다며 설명을 덧붙였습니다. 화재 이후 어린 정원 씨를 거두어 키워 준 이모가 몇 해 전 세상을 떠나면서, 유품을 정리하던 친척들이 이모의 오래된 옷가지들을 자선단체에 통째로 기증했는데, 그 코트가 바로 그중 하나였을 것이라고 했습니다. 코트 안주머니에 테이프가 들어 있는 줄은, 정원 씨 자신도 전혀 모르고 있었습니다.[PAUSE]정옥 씨는 조심스럽게 물었습니다. "이모님 유품인 줄 모르고 넘겨 드렸다니, 혹시 서운하게 들리시진 않으셨어요." 정원 씨는 고개를 저으며 나직이 웃었습니다. "아니요. 오히려 다행이에요. 이모가 마지막까지 이걸 소중히 걸어 두셨던 거잖아요. 잃어버렸다고 생각했던 게, 이렇게 돌아왔으니까요."[PAUSE]정원 씨는 잠시 창밖을 바라보다가, 다시 정옥 씨 쪽으로 몸을 돌렸습니다. "사실 저는 어머니 목소리가 어땠는지도 가물가물했어요. 사진 한 장 없으니까, 시간이 지날수록 얼굴도 목소리도 점점 흐려지더라고요. 그런데 아까 잠깐 튼 부분에서, 어머니가 제 이름을 부르는 그 억양이, 듣자마자 그냥 온몸에 소름이 돋았습니다. 이게 진짜 우리 엄마구나, 하고요." 정옥 씨는 그 말을 들으며 자신도 모르게 눈시울이 붉어지는 것을 느꼈습니다.[PAUSE]정원 씨는 테이프를 두 손으로 꼭 쥔 채 한동안 말을 잇지 못하다가, 문득 정옥 씨에게 물었습니다. "이걸 찾으시려고, 규정까지 어기면서 애쓰셨다고 들었어요. 저한테는 이게 세상 전부인 물건이지만, 정옥 씨한테는 그냥 낡은 카세트테이프 하나였을 텐데, 왜 그렇게까지 하셨어요." 정옥 씨는 잠시 생각하다가 담담히 대답했습니다. "저도 잘 모르겠어요. 그냥, 이걸 그대로 부숴 버리면 다시는 되돌릴 수 없다는 게, 마음에 걸려서요."[PAUSE]정옥 씨가 사무실로 돌아와 이 일을 박 팀장에게 보고하자, 박 팀장은 잠시 말이 없다가 짧게 한숨을 내쉬었습니다. "정옥 씨, 규정은 규정이니 경고 기록은 그대로 남을 겁니다. 그건 저도 어쩔 수 없어요." 정옥 씨는 담담하게 고개를 끄덕였습니다. "괜찮습니다. 저는 이제 곧 나갈 사람인걸요." 박 팀장은 그 말에 잠시 정옥 씨를 바라보다가, "수고하셨습니다"라는 말을 짧게 남기고 자리를 떴습니다.[PAUSE]정옥 씨의 정년퇴직일이 마침내 다가왔습니다. 특별한 행사도, 꽃다발도 없이, 정옥 씨는 여느 날과 다름없이 아침 일찍 출근해 마지막으로 창구에 앉았습니다. 그날따라 분실물 신고가 유난히 많았고, 정옥 씨는 우산 세 개와 지갑 하나, 그리고 아이의 장갑 한 짝을 각각의 주인에게 돌려주었습니다.[PAUSE]퇴근 시간이 되어 짐을 정리하던 정옥 씨는, 서랍 맨 아래 칸에서 그동안 미처 주인을 찾지 못했던 작은 물건들의 사진을 모아 둔 낡은 수첩을 발견했습니다. 단추 하나, 빛바랜 사진 한 장, 이름 모를 열쇠 하나. 정옥 씨는 그 수첩을 버리지 않고, 조용히 가방 안에 챙겨 넣었습니다.[PAUSE]정옥 씨는 사무실을 나서기 전, 텅 빈 유실물 선반을 한 번 더 둘러보았습니다. 마흔두 해 동안 이 선반을 거쳐 간 무수한 물건들, 그리고 그 물건들 뒤에 숨어 있던 사람들의 사연이 스쳐 지나갔습니다. 정옥 씨는 문득, 자신이 이 일에서 배운 것은 대단한 기술이나 요령이 아니라, 남들이 하찮게 여기고 지나칠 법한 작은 것에 오래 눈길을 두는 태도였다는 것을 깨달았습니다.[PAUSE]정옥 씨는 후배들에게 무언가를 가르치거나 물려줄 생각은 하지 않았습니다. 다만 나가는 길에, 선반 옆 게시판에 붙어 있던 낡은 안내문 한 줄을 손수 고쳐 적었을 뿐입니다. "폐기 전, 다시 한번 들여다보기." 그것은 후임자를 위한 지침이라기보다, 마흔두 해 동안 정옥 씨 자신이 스스로에게 다짐해 온 말을 마지막으로 남겨 두는 것에 더 가까웠습니다.[PAUSE]며칠 뒤, 정옥 씨의 집으로 작은 소포 하나가 도착했습니다. 발신인은 강정원 씨였습니다. 소포 안에는 그 카세트테이프를 복원해 만든 디지털 음원 파일이 담긴 손바닥만 한 저장 장치와, 짧은 편지 한 장이 들어 있었습니다. "덕분에 어머니 목소리를 다시 들을 수 있게 됐습니다. 이제 이 목소리는 저 혼자만의 것이 아니라, 언젠가 제 아이에게도 들려줄 수 있는 것이 되었습니다. 정옥 씨가 아니었다면, 이 목소리는 정말로 사라졌을 겁니다."[PAUSE]오늘 밤의 이야기는 여기서 마치겠습니다. 정옥 씨가 마흔두 해 동안 지켜 온 것은, 크고 화려한 무언가가 아니라 남들이 쉽게 버리고 지나칠 작은 물건 하나에 담긴 마음을 끝까지 놓지 않는 태도였습니다. 편안한 마음으로, 부디 오늘 밤도 푹 주무시길 바랍니다. 좋은 꿈 꾸시고, 안녕히 주무세요.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>こんにちは。お昼の脳トレクイズの時間です。今日は、日本と韓国、それぞれの昔話にまつわる問題を五つご用意しました。子どもの頃に聞いた話を思い出しながら、一緒に考えてみてくださいね。どちらの国のお話も、長い年月を経て今に伝えられてきた、大切な文化の一つです。[PAUSE]最初の問題です。おじいさんが川で拾った大きな桃から生まれた男の子は、何という名前で知られているでしょうか。[PAUSE]正解は「桃太郎」です。犬、猿、雉を家来にして鬼退治に向かう物語は、日本の昔話の中でも特に広く知られています。きびだんごを分け与える場面を覚えている方も多いのではないでしょうか。地域によっては、桃太郎の出身地を名乗る土地がいくつも存在し、それぞれに独自の言い伝えが残っているのも興味深いところです。[PAUSE]二問目です。韓国の昔話で、木こりが天女の羽衣を隠して結婚したという伝承は、一般に何という物語として知られているでしょうか。[PAUSE]正解は「ソンニョと木こり」、日本語では「天女の羽衣」に近い物語として紹介されることもあります。天に帰りたい天女と、それを引き止める木こりの切ない物語で、地域によって結末が異なる伝承も残っているのだそうです。日本各地にも同じように、天から舞い降りた乙女が羽衣を奪われて地上に留まるという、似た構造を持つ伝説が数多く伝わっています。[PAUSE]三問目です。日本の昔話で、おばあさんが川で洗濯をしていると、川上から流れてきた大きなものといえば何でしょうか。[PAUSE]正解は「桃」です。「おじいさんは山へ柴刈りに、おばあさんは川へ洗濯に」という、あの有名な語り出しの続きにあたる場面ですね。[PAUSE]四問目です。韓国の昔話「フンブとノルブ」で、心優しい弟が助けたのは、足を痛めたどんな生き物だったでしょうか。[PAUSE]正解は「つばめ」です。弟フンブが足を折ったつばめを助けたことで幸運を授かり、逆に強欲な兄ノルブが真似をして痛い目にあうという、勧善懲悪の物語として親しまれています。[PAUSE]最後の問題です。日本の昔話「浦島太郎」で、主人公が竜宮城から持ち帰った、決して開けてはいけないと言われた箱は何と呼ばれているでしょうか。[PAUSE]正解は「玉手箱」です。開けた途端に煙が立ちのぼり、太郎は一気に年をとってしまう、という結末を覚えている方も多いことでしょう。決して開けるなと言われたものほど気になってしまうのは、昔も今も変わらない人の性なのかもしれません。[PAUSE]五問とも、いかがでしたでしょうか。日本と韓国、それぞれの土地で語り継がれてきた昔話には、動物への優しさや、約束を守ることの大切さなど、共通する教えが多く込められているように感じます。国は違っても、大切にしてきた心はどこか似ているものなのかもしれません。今日はどちらの国のお話が印象に残りましたか。お孫さんやお子さんに、今日覚えたお話を聞かせてあげるのも良いかもしれませんね。それでは、また明日のクイズでお会いしましょう。今日も最後までありがとうございました。</t>
+          <t>こんにちは。お昼の脳トレクイズの時間です。今日は、日本と韓国の昔話から、少しずつ難しくなる五問を用意しました。同じ物語を重ねず、五つの異なる世界を旅します。答えを急がず、子どもの頃に聞いた場面を思い浮かべてくださいね。[PAUSE]第一問。日本の昔話で、桃から生まれ、犬・猿・雉と鬼退治へ向かった主人公は誰でしょう。金太郎、桃太郎、浦島太郎、一寸法師から選んでください。[PAUSE]正解は「桃太郎」です。仲間にきびだんごを分け、一緒に困難へ向かう姿が長く語り継がれてきました。岡山をはじめ物語ゆかりの地を名乗る地域が複数あり、土地ごとに少し違う伝承を味わえるのも面白いところです。[PAUSE]第二問。韓国の「フンブとノルブ」で、心優しい弟フンブが手当てをした生き物は何でしょう。つばめ、うさぎ、亀、鶴から選んでください。[PAUSE]正解は「つばめ」です。元気になったつばめが運んだ種から大きな瓢箪が実り、フンブへ幸運をもたらします。一方、欲から同じことをまねた兄ノルブには災いが訪れます。親切と欲の違いが、二人の兄弟を通してはっきり描かれています。[PAUSE]第三問。竹の中から光とともに現れ、やがて月へ帰る日本の物語の主人公は誰でしょう。かぐや姫、乙姫、鶴女房、織姫から選んでください。[PAUSE]正解は「かぐや姫」です。「竹取物語」は日本最古の物語文学とされ、求婚者たちへ難題を出す場面や、育ての親との別れまで多くの人の心に残っています。美しいだけでなく、自分の意思を持つ主人公として読み直してみるのも興味深いですね。[PAUSE]第四問。韓国の「コンジとパッチ」で、働き者のコンジを助ける生き物の一つはどれでしょう。牛、狐、鶴、虎の四つから選んでください。[PAUSE]正解は「牛」です。伝承には異なる形もありますが、牛やひきがえるなどが難しい仕事を助ける場面がよく知られています。つらい状況でも誠実さを失わないコンジに、自然の存在が力を貸すところが印象的です。[PAUSE]最後の問題です。浦島太郎が竜宮城から持ち帰り、開けてはいけないと言われた箱は何でしょう。宝手箱、玉手箱、竜宮箱、乙姫箱から選んでください。[PAUSE]正解は「玉手箱」です。箱を開けると白い煙が立ちのぼり、太郎はたちまち年老いてしまいます。助けた亀に導かれた華やかな竜宮城と、戻った故郷で長い時が過ぎていた寂しさ。その対比が、時間と約束をめぐる不思議で少し切ない余韻を残します。[PAUSE]五問すべて終わりました。いくつ正解できましたか。日本と韓国の昔話には、親切が巡って戻ること、欲に流されないこと、約束の重さなど、国を越えて響き合う教えがあります。正解の数だけでなく、忘れていた場面を一つ思い出せたなら、それも今日の立派な成果です。家族と答えを比べたり、知っている別の結末を話したりすれば、記憶はさらに生き生きしてきます。五問の中から一つ選び、登場人物の立場なら自分はどうするか考えてみるのも、よい脳の運動になります。それでは、また明日のクイズでお会いしましょう。最後までありがとうございました。</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>町の外れの、少し坂道を上ったところに、昭和の頃から続く小さな銭湯がありました。その番台に座り続けて四十年になる清子さんが、体調を崩して初めて店を休んだあの冬の日から、今夜の物語は始まります。[PAUSE]こんばんは。今夜も、こもれび便りに、こうしてお付き合いいただき、ありがとうございます。どうぞ肩の力を抜いて、ゆっくりとお聞きください。[PAUSE]清子さんは、若い頃から夫と二人三脚でこの銭湯を切り盛りしてきましたが、夫を十年前に病気で亡くしてからは、寂しさを抱えながらも一人で番台に座り続けていました。常連客一人一人の顔と名前をすべて覚え、誰がどんな湯加減を好むかまで、すべて把握しているほど、清子さんはまさにこの銭湯そのものでした。町の高齢者たちにとって、毎日の入浴は、ただ体を清めるだけでなく、清子さんとの短い会話をゆっくり楽しむ、大切な日課でもありました。[PAUSE]ある冬の朝、清子さんは高熱を出して起き上がれなくなりました。駆けつけた医者からは、無理をしすぎた体をしっかりと休ませるため、しばらくの静養が必要だと言い渡されました。清子さんには、遠方で働く一人娘の美咲がいましたが、美咲は仕事の都合で、すぐには帰ってこられない事情がありました。銭湯を臨時休業にするしかないと諦めかけたとき、美咲は電話越しに意外な提案をしました。「お母さん、私、少しの間、番台に座ってみようかな」。[PAUSE]美咲は、幼い頃から番台のそばで宿題をしたり、脱衣所の掃除を手伝ったりして育ちましたが、大人になってからは町を離れ、番台に座ったことなど一度もありませんでした。それでも、母が大切にしてきた場所を閉めたままにはしたくないという一心で、急遽休暇を取り、実家に戻ってきました。美咲は、清子さんの布団の脇に座り、番台の仕事について一から教えてもらうことにしました。[PAUSE]しかし、実際に番台に座ってみると、思っていた以上に勝手が分かりませんでした。常連客の名前も顔もほとんど覚えておらず、料金のやり取りや脱衣所の管理にも戸惑うばかりです。ある常連の男性客から、「いつもの清子さんはどうしたんだ」と怪訝な顔をされ、美咲は言葉に詰まってしまいました。母の不在を寂しく思う客の気持ちが、痛いほど伝わってきたからです。[PAUSE]美咲は次の日も緊張した面持ちで朝早くから番台に座りましたが、脱衣所の鍵の掛け方や、常連客ごとに違うタオルの置き場所など、細かなことでも次々とつまずきました。ある年配の女性客からは、「新しい人には慣れないだろうけど、頑張ってね」と励まされる一方で、勝手の違いに戸惑う美咲自身の不慣れさを見透かされているようで、情けない気持ちにもなりました。[PAUSE]その日の夜、美咲は借りた布団の中で泣きそうになりながら、母にその日の出来事を話しました。清子さんは布団に横たわったまま、しばらく黙って静かに耳を傾けたあと、「お客さん一人一人の顔と名前を、焦らず少しずつ覚えていけばいい。私も最初はそうだったから」と、優しく声をかけてくれました。美咲は、母がこの四十年間、当たり前のように積み重ねてきたことの重みを、初めて実感しました。[PAUSE]美咲は、以前勤めていた営業の仕事で身につけた、相手をよく観察し、小さな変化も見逃さないという習慣をふと思い出しました。仕事では顧客の好みや要望を細かくメモして関係を築いてきましたが、その方法を番台の仕事にも応用できるのではないかと考えたのです。美咲はさっそく、脱衣所の隅にほこりをかぶって置いてあった古い帳面を手に取り、そこに気づいたことを書き留め始めました。[PAUSE]翌日から、美咲は客が来るたびに、その日のうちに小さな手帳にその人の特徴と名前を書き留めるようになりました。杖をついた元気な田中のおじいさん、いつも赤ちゃんを連れてくる若いお母さん、無口だけれど風呂上がりに必ず牛乳を飲む中年の男性。美咲は一人一人との短いやり取りを大切にしながら、少しずつ常連客の顔を覚えていきました。[PAUSE]実は、清子さんの夫、つまり美咲の父は、生前、機械いじりが得意な人でした。近所の電気屋に頼めば済むような簡単な修理でも、自分の手でやってみたがる性格で、そのぶん銭湯の設備には人一倍愛着を持っていたと、美咲は幼い頃の記憶をたどりながら思い出していました。その頃、美咲はふと、亡くなった父のことを思い出していました。生前、父はよくボイラー室で無口に機械の手入れをしていて、母がその横で客と談笑する声が響いていたものです。父が担っていた裏方の仕事のことまで、母が一人でこなしていたのだと気づき、美咲は改めて母の苦労の大きさを実感しました。一週間ほど経った頃、清子さんの熱はようやく下がり始めましたが、まだ本調子ではありませんでした。美咲はこのまま自分の仕事に戻るべきか、もう少し母のそばにいるべきか、番台に座りながら何度も思い悩んでいました。そんなとき、常連客の一人である田中さんが、番台に座る美咲に声をかけてきました。「あんた、だいぶ様になってきたな。清子さんも、きっと安心してるよ」。[PAUSE]田中さんはさらに、こんな話もしてくれました。「わしがここに通い始めたのは、女房を亡くした年でな。毎日誰とも話さない日が続いて、気が滅入っていたんだ。でも、この番台で清子さんと少し話すだけで、なんだか救われる気がしてなあ」。美咲は、番台という場所が、単なる料金のやり取りの場ではなく、人と人との心のつながりを支える場所なのだと、改めて実感しました。田中さんのその言葉に、美咲は胸が熱くなりました。これまで気づかなかった、番台という仕事の奥深さと温かさを、身をもって感じるようになっていたのです。美咲は上司に丁寧に事情を説明し、有給休暇を延長してもらい、母が完全に回復するまで、この場所を自分の手でしっかりと守り続けることに決めました。[PAUSE]ちょうどその頃、銭湯にとってさらに困った出来事が重なりました。長年使ってきたボイラーが老朽化により不調を起こし、駆けつけた修理業者からは、部品がすでに製造中止になっており、修理には想像以上の時間もお金もかなりかかると告げられたのです。美咲は母に代わってその対応にも追われることになり、慣れない番台の仕事に加えて、大きな決断まで任されることになってしまいました。[PAUSE]美咲はその日のうちに複数の業者から見積もりを取り寄せ、慣れない専門用語と格闘しながら、修理か、それとも新しいボイラーへの交換かで悩みました。交換となれば、貯金のほとんどを使い果たすことになります。清子さんは布団の中から、「もう潮時かもしれない。無理して続けることはないよ」と力なく言いました。長年の疲れも重なり、母がこの機会に店を畳むことを考え始めていることが、美咲には痛いほど伝わってきました。[PAUSE]しかし美咲は、この一週間で見てきた常連客たちの顔を思い浮かべました。杖をついて毎日通う田中さん、赤ちゃんを連れてくる若い母親、無口だけれど必ず顔を出す中年の男性。この銭湯がなくなれば、彼らの日課そのものが失われてしまう。美咲は思い切って、自分の貯金を取り崩し、新しいボイラーへの交換に踏み切ることを母に提案しました。[PAUSE]清子さんは、「そんな大金、娘に出させるわけにはいかない」と強く反対しましたが、美咲は「これは、私がこの三週間で学んだことへの恩返しだから」と譲りませんでした。押し問答の末、清子さんはようやく折れ、美咲の申し出を受け入れることにしました。工事の間、銭湯は一週間の臨時休業を余儀なくされましたが、常連客たちは口々に「待ってるから、ゆっくりやって」と温かい言葉をかけてくれました。休業中、美咲は毎日工事の様子を見に通い、慣れない専門用語に戸惑いながらも、業者とのやり取りや進捗の確認を一手に引き受けました。工事が完了した再開初日、田中さんをはじめとする常連客たちが次々と詰めかけ、「新しい湯船は気持ちいいねえ」と口々に喜びの声を上げました。[PAUSE]美咲が番台に座り続けるうちに、常連客たちも彼女に少しずつ心を開いていきました。ある日、いつも無口な男性客が、珍しく美咲に話しかけてきました。「俺は妻を亡くしてから、この銭湯だけが唯一の楽しみなんだ。清子さんも、あんたも、ここに座っていてくれるだけで、こっちは救われるんだよ」。美咲は、その言葉に深く胸を打たれました。[PAUSE]ある日、若い世代がこの仕事に興味を持ってくれることはないだろうかと、美咲はふと考えることがありました。近所の高校生が、部活帰りに銭湯を覗き込み、珍しそうに番台を眺めていく姿を見かけたのがきっかけでした。美咲は声をかけ、「よかったら、たまに手伝ってみない?」と誘ってみましたが、その高校生は照れくさそうに笑って去っていきました。それでも美咲は、いつかこの場所に、また新しい若い力が加わる日が来るかもしれないと、密かに期待を抱くようになりました。[PAUSE]三週間後、清子さんはようやく体力を取り戻し、久しぶりに番台に戻ってきました。美咲は横に座り、清子さんが常連客たちと再会する様子を見守りました。「清子さん、待ってたよ」「元気になってよかった」。次々とかけられる温かい言葉に、清子さんは涙ぐみながら、深々と頭を下げていました。[PAUSE]帰りの荷造りをしながら、美咲はこの三週間の出来事を振り返り、まさか自分がこんなにも銭湯の仕事に心を動かされるとは思ってもみなかったと、一人静かに驚いていました。その夜、美咲は東京へ戻る支度をしながら、清子さんに切り出しました。「お母さん、私、月に一度でいいから、また帰ってきて番台に座らせてもらえないかな。すごく、大切な時間だったから」。清子さんは驚きながらも、嬉しそうに頷きました。それから美咲は、月に一度、実家に帰っては番台に座る生活を続けるようになりました。[PAUSE]月に一度の帰省が始まってから一年ほど経った頃、美咲は東京の職場で大きな昇進の話を持ちかけられました。海外支社への異動を伴う昇進で、これを受ければ、これまでのように月に一度実家に帰ることも難しくなります。美咲は、これまで積み上げてきたキャリアと、銭湯での大切な時間との間で、深く思い悩むことになりました。[PAUSE]美咲は上司に少し考えさせてほしいと伝え、次の帰省の際、清子さんにこの話を打ち明けました。清子さんは黙って話を聞いたあと、「あなたの人生よ。私のことは気にしなくていい。銭湯は、いつか閉めることになっても仕方ないんだから」と、寂しさを押し殺すように言いました。その言葉とは裏腹に、清子さんの目には隠しきれない切なさがにじんでいました。[PAUSE]その晩、美咲は眠れないまま、番台に一人座ってみました。閉店後の静まり返った浴室に、かつて聞いた常連客たちの声がよみがえってきます。「清子さんも、あんたも、ここに座っていてくれるだけで、こっちは救われるんだよ」。あの無口な男性客の言葉が、繰り返し頭の中に響きました。美咲は、この場所が自分にとってもかけがえのないものになっていることに、改めて気づかされました。[PAUSE]眠れないまま迎えた朝、美咲は洗面所の鏡に映る自分の顔を見つめ、これまでの数年間で自分がどれほど変わったかを実感しました。東京で働いていた頃には見えなかった、人と人との細やかなつながりの尊さに、この銭湯を通じて気づかされていたのです。翌朝、美咲は昇進の話を丁重に断ることに決めました。上司には、家庭の事情があると正直に伝え、代わりに国内での別の役職に就かせてもらえないか相談しました。上司は少し驚いた様子でしたが、美咲の真剣な表情を見て、「そこまで大切に思える場所があるのは、うらやましいことだよ」と言い、希望を聞き入れてくれました。[PAUSE]決断を伝える前夜、美咲は東京の静かな自分の部屋で一人、これまで築いてきたキャリアの重みと、銭湯で過ごした短い日々の温かさを、天秤にかけるように何度も考え直していました。特に親しくしていた先輩からは「せっかくここまで積み上げてきたのに」と心配され、他の同僚たちからも「もったいない」と惜しまれるだろうことも分かっていましたが、番台に座って感じたあの充足感に勝るものはないという確信だけは、揺らぐことがありませんでした。美咲がその決断を清子さんに伝えると、清子さんは驚きながらも、「無理はしないでほしい」と繰り返しました。美咲は首を横に振り、「無理をしているんじゃないの。ここが、私の大切な場所になったから、選んだだけ」と答えました。清子さんは、それ以上何も言わず、ただ静かに美咲の手を握りしめました。[PAUSE]それから美咲は、以前よりも頻繁に実家に帰るようになり、清子さんの体調が思わしくない日には、数日間泊まり込んで番台に座ることも増えていきました。常連客たちも、美咲が定期的に顔を出すことを当たり前のように受け止め、時には清子さんよりも先に、美咲に世間話を持ちかける客も出てくるようになりました。[PAUSE]数年後、清子さんが体力的に銭湯を続けるのが難しくなったとき、美咲は東京での仕事に区切りをつけ、正式に実家に戻って銭湯を継ぐことを決意しました。あの三週間で覚えた常連客たちの顔と名前は、すでに美咲の中でしっかりと根を張っていました。正式に番台を引き継ぐ日、清子さんは長年愛用してきた古い座布団を美咲に手渡しました。座布団の裏地には何度も繕われた跡があり、長い年月を物語っていました。「これに座って、初めてお客さんの顔をちゃんと見られるようになったの」と、清子さんは懐かしそうに目を細めました。清子さんは、番台を美咲に譲る日、静かにこう言いました。「この仕事は、体を洗う手伝いをするだけじゃない。人の暮らしに、ほんの少し寄り添う仕事なんだよ」。[PAUSE]美咲が正式に銭湯を継いでから二年ほど経った頃、思いがけない知らせが届きました。町の再開発計画により、銭湯のある一帯が数年以内に区画整理の対象になるかもしれないというのです。美咲は役所からの説明会に足を運び、詳しい事情を確認しました。計画が実行されれば、銭湯の建物も立ち退きの対象になる可能性があるとのことでした。[PAUSE]美咲はこの話を聞いて、目の前が真っ暗になるような気持ちを味わいました。せっかく母から受け継ぎ、常連客たちとの絆を築いてきたこの場所が、行政の計画一つで失われてしまうかもしれない。美咲は居ても立ってもいられず、同じように影響を受ける近隣の商店主たちと連絡を取り合い、対策を考える集まりを開くことにしました。[PAUSE]集まりには、長年この商店街で店を構えてきた人々が次々と参加しました。美咲は、銭湯が単なる入浴施設ではなく、高齢者たちの見守りの場、地域の交流の場としての役割を果たしていることを、これまでの経験をもとに説明しました。参加者たちは、それぞれの店が持つ地域での役割について語り合い、行政に対して再開発計画の見直しを求める要望書をまとめることになりました。[PAUSE]要望書の作成にあたり、美咲は自分の手帳に書き留めてきた常連客たちの記録を活用することにしました。誰が何年通っているか、銭湯がどんな役割を果たしてきたか、具体的な数字と共に文書にまとめていきました。田中さんをはじめとする常連客たちも、自ら役所に足を運び、直接自分たちの思いを伝えてくれました。[PAUSE]話し合いの中で、行政の担当者は当初、地域の意見をあまり重視しない姿勢を見せていましたが、美咲たちが粘り強く何度も足を運び、実際の利用状況や高齢者たちの声を届け続けるうちに、次第にその態度も軟化していきました。ある担当者は、「これほど地域に根ざした場所だとは、正直、想像していませんでした」と率直に語り、住民側の主張に理解を示すようになりました。数ヶ月にわたる話し合いの末、行政側は計画を全面的に見直し、銭湯を含む一角については、再開発の対象から除外するという決定を下しました。説明会の場で、この結果を聞いた美咲は、思わずその場に座り込みそうになるほどの安堵を覚えました。田中さんは美咲の肩を叩き、「あんたが頑張ってくれたおかげだ」と、目を潤ませながら言いました。[PAUSE]要望書をまとめる過程で、美咲は普段あまり関わりのなかった隣の惣菜屋の店主や、向かいのクリーニング店の若い店主とも、初めてじっくり言葉を交わす機会を得ました。それぞれが抱える悩みは違っていても、地域の人々を支えたいという思いは共通していることに気づき、美咲はこの商店街全体が、目に見えない形で支え合っていたのだと実感しました。この出来事をきっかけに、美咲は商店街の若手経営者たちとのつながりを深め、月に一度の情報交換会を自ら呼びかけて始めるなど、地域全体で高齢者を支える緩やかなネットワークづくりにも関わるようになりました。銭湯という一つの場所を守るために始めた行動が、思いがけず町全体を巻き込む大きな動きへとつながっていったのです。美咲は今も、あの手帳を大切に手元に置いています。新しい客が来るたびに、名前と特徴を書き足しながら、清子さんが四十年かけて築いてきたものを、少しずつ自分の手で育て直しているのです。白い湯気の立ちのぼる銭湯の向こうには、今日もたくさんの顔なじみが、いつも変わらぬ笑顔で美咲を迎えてくれます。[PAUSE]銭湯が存続することになったあの年の冬、清子さんは静かに息を引き取りました。最期の時、清子さんは病室から美咲の手を握り、「あなたが継いでくれて、本当によかった」と、かすれた声で伝えました。葬儀には、田中さんをはじめとする常連客たちが数多く参列し、清子さんとの思い出を涙ながらに語り合いました。[PAUSE]母を失った悲しみの中でも、美咲は毎日欠かさず番台に座り続けました。悲しみに沈んでいる暇はないというよりも、番台に座り、常連客たちと言葉を交わすことこそが、美咲にとって一番の慰めになっていたのです。ある日、いつもの無口な男性客が、珍しく長く話し込んでいきました。「清子さんも、きっとこの湯気の向こうから見てるよ」。その一言に、美咲は静かに涙をこぼしました。[PAUSE]銭湯を一人で切り盛りする日々の中で、美咲は自分の体力の限界も感じるようになっていました。朝早くから夜遅くまでボイラーの管理から番台、清掃までをすべて一人でこなすのは、想像以上に重労働でした。ある晩、美咲は疲れ果てて番台に突っ伏したまま眠り込んでしまい、翌朝、早くに来た常連の女性客に心配されて起こされるということもありました。「一人で全部背負い込まなくていいのよ」。その女性客の言葉が、美咲の胸に深く残りました。[PAUSE]母の死から半年ほど経ったある日、美咲のもとに、遠方に住む親戚から思いがけない相談が寄せられました。親戚の息子である健太という青年が、就職先が決まらず将来に悩んでいるので、しばらく銭湯の手伝いをさせてもらえないかというのです。美咲は、かつての自分自身と重ねながら、快く健太を受け入れることにしました。[PAUSE]健太は色白で物静かな青年で、人前に立つと緊張のあまり言葉が詰まってしまう性格でしたが、面接ではうまく自分を表現できず、いくつもの会社から立て続けに不採用の通知を受け取っていました。両親からも「もっと積極的にならないと」と言われ続け、すっかり自信を失っていました。美咲は、あえて仕事の細かい指示を多く出さず、まずは常連客たちとの何気ない会話に慣れてもらうことから始めました。最初はぎこちなかった健太も、田中さんに冗談を返されて思わず笑ってしまうなど、少しずつ肩の力が抜けていく様子が見て取れました。健太は最初こそ慣れない仕事に戸惑いながらも、美咲の丁寧な指導のもと、少しずつ番台の仕事を覚えていきました。美咲は、かつて清子さんが自分にしてくれたように、焦らず一人一人の常連客の顔と名前を覚えるよう、根気強く健太に教えました。あの手帳は、こうして三代目の記録として、新しいページが加えられていくことになったのです。[PAUSE]ある日、健太が思い切って美咲にこう打ち明けました。「正直、最初はただの腰かけのつもりでした。でも、常連さんたちが名前を覚えて声をかけてくれるようになって、自分が誰かに必要とされてるって実感が持てたんです」。美咲は、その言葉を聞きながら、かつて自分自身が抱いた思いと重なる部分に、深くうなずきました。健太は半年ほど手伝ううちに、それまでの弱気な表情が嘘のように明るくなり、この仕事に本気で向き合いたいという気持ちを固め、正式に銭湯で働かせてほしいと美咲に申し出ました。美咲はその申し出を喜んで受け入れ、いずれは健太にも、この場所の大切さを引き継いでいってほしいと願うようになりました。清子さんから美咲へ、そして美咲から健太へと、番台に込められた思いは、静かに、しかし確かに受け継がれていったのです。[PAUSE]急な、思いがけない出来事がきっかけで、誰かの大切な場所を引き継ぐことになる。そんなとき、大きな不安や戸惑いの中にも、これまで気づかなかった大切な尊さが隠れていることがあるのかもしれません。今夜の長いお話は、ここまでです。どうか安心して、今夜もゆっくりとお休みください。良い夢を。ゆっくり、おやすみなさい。</t>
+          <t>町の外れの、少し坂道を上ったところに、昭和の頃から続く小さな銭湯がありました。その番台に座り続けて四十年になる清子さんが、体調を崩して初めて店を休んだあの冬の日から、今夜の物語は始まります。[PAUSE]こんばんは。今夜も、こもれび便りに、こうしてお付き合いいただき、ありがとうございます。どうぞ肩の力を抜いて、ゆっくりとお聞きください。[PAUSE]清子さんは、若い頃から夫と二人三脚でこの銭湯を切り盛りしてきましたが、夫を十年前に病気で亡くしてからは、寂しさを抱えながらも一人で番台に座り続けていました。常連客一人一人の顔と名前をすべて覚え、誰がどんな湯加減を好むかまで、すべて把握しているほど、清子さんはまさにこの銭湯そのものでした。町の高齢者たちにとって、毎日の入浴は、ただ体を清めるだけでなく、清子さんとの短い会話をゆっくり楽しむ、大切な日課でもありました。[PAUSE]ある冬の朝、清子さんは高熱を出して起き上がれなくなりました。駆けつけた医者からは、無理をしすぎた体をしっかりと休ませるため、しばらくの静養が必要だと言い渡されました。清子さんには、遠方で働く一人娘の美咲がいましたが、美咲は仕事の都合で、すぐには帰ってこられない事情がありました。銭湯を臨時休業にするしかないと諦めかけたとき、美咲は電話越しに意外な提案をしました。「お母さん、私、少しの間、番台に座ってみようかな」。[PAUSE]美咲は、幼い頃から番台のそばで宿題をしたり、脱衣所の掃除を手伝ったりして育ちましたが、大人になってからは町を離れ、番台に座ったことなど一度もありませんでした。それでも、母が大切にしてきた場所を閉めたままにはしたくないという一心で、急遽休暇を取り、実家に戻ってきました。美咲は、清子さんの布団の脇に座り、番台の仕事について一から教えてもらうことにしました。[PAUSE]しかし、実際に番台に座ってみると、思っていた以上に勝手が分かりませんでした。常連客の名前も顔もほとんど覚えておらず、料金のやり取りや脱衣所の管理にも戸惑うばかりです。ある常連の男性客から、「いつもの清子さんはどうしたんだ」と怪訝な顔をされ、美咲は言葉に詰まってしまいました。母の不在を寂しく思う客の気持ちが、痛いほど伝わってきたからです。[PAUSE]美咲は次の日も緊張した面持ちで朝早くから番台に座りましたが、脱衣所の鍵の掛け方や、常連客ごとに違うタオルの置き場所など、細かなことでも次々とつまずきました。ある年配の女性客からは、「新しい人には慣れないだろうけど、頑張ってね」と励まされる一方で、勝手の違いに戸惑う美咲自身の不慣れさを見透かされているようで、情けない気持ちにもなりました。[PAUSE]その日の夜、美咲は借りた布団の中で泣きそうになりながら、母にその日の出来事を話しました。清子さんは布団に横たわったまま、しばらく黙って静かに耳を傾けたあと、「お客さん一人一人の顔と名前を、焦らず少しずつ覚えていけばいい。私も最初はそうだったから」と、優しく声をかけてくれました。美咲は、母がこの四十年間、当たり前のように積み重ねてきたことの重みを、初めて実感しました。[PAUSE]美咲は、以前勤めていた営業の仕事で身につけた、相手をよく観察し、小さな変化も見逃さないという習慣をふと思い出しました。仕事では顧客の好みや要望を細かくメモして関係を築いてきましたが、その方法を番台の仕事にも応用できるのではないかと考えたのです。美咲はさっそく、脱衣所の隅にほこりをかぶって置いてあった古い帳面を手に取り、そこに気づいたことを書き留め始めました。[PAUSE]翌日から、美咲は客が来るたびに、その日のうちに小さな手帳にその人の特徴と名前を書き留めるようになりました。杖をついた元気な田中のおじいさん、いつも赤ちゃんを連れてくる若いお母さん、無口だけれど風呂上がりに必ず牛乳を飲む中年の男性。美咲は一人一人との短いやり取りを大切にしながら、少しずつ常連客の顔を覚えていきました。[PAUSE]実は、清子さんの夫、つまり美咲の父は、生前、機械いじりが得意な人でした。近所の電気屋に頼めば済むような簡単な修理でも、自分の手でやってみたがる性格で、そのぶん銭湯の設備には人一倍愛着を持っていたと、美咲は幼い頃の記憶をたどりながら思い出していました。その頃、美咲はふと、亡くなった父のことを思い出していました。生前、父はよくボイラー室で無口に機械の手入れをしていて、母がその横で客と談笑する声が響いていたものです。父が担っていた裏方の仕事のことまで、母が一人でこなしていたのだと気づき、美咲は改めて母の苦労の大きさを実感しました。一週間ほど経った頃、清子さんの熱はようやく下がり始めましたが、まだ本調子ではありませんでした。美咲はこのまま自分の仕事に戻るべきか、もう少し母のそばにいるべきか、番台に座りながら何度も思い悩んでいました。そんなとき、常連客の一人である田中さんが、番台に座る美咲に声をかけてきました。「あんた、だいぶ様になってきたな。清子さんも、きっと安心してるよ」。[PAUSE]田中さんはさらに、こんな話もしてくれました。「わしがここに通い始めたのは、女房を亡くした年でな。毎日誰とも話さない日が続いて、気が滅入っていたんだ。でも、この番台で清子さんと少し話すだけで、なんだか救われる気がしてなあ」。美咲は、番台という場所が、単なる料金のやり取りの場ではなく、人と人との心のつながりを支える場所なのだと、改めて実感しました。田中さんのその言葉に、美咲は胸が熱くなりました。これまで気づかなかった、番台という仕事の奥深さと温かさを、身をもって感じるようになっていたのです。美咲は上司に丁寧に事情を説明し、有給休暇を延長してもらい、母が完全に回復するまで、この場所を自分の手でしっかりと守り続けることに決めました。[PAUSE]ちょうどその頃、銭湯にとってさらに困った出来事が重なりました。長年使ってきたボイラーが老朽化により不調を起こし、駆けつけた修理業者からは、部品がすでに製造中止になっており、修理には想像以上の時間もお金もかなりかかると告げられたのです。美咲は母に代わってその対応にも追われることになり、慣れない番台の仕事に加えて、大きな決断まで任されることになってしまいました。[PAUSE]美咲はその日のうちに複数の業者から見積もりを取り寄せ、慣れない専門用語と格闘しながら、修理か、それとも新しいボイラーへの交換かで悩みました。交換となれば、貯金のほとんどを使い果たすことになります。清子さんは布団の中から、「もう潮時かもしれない。無理して続けることはないよ」と力なく言いました。長年の疲れも重なり、母がこの機会に店を畳むことを考え始めていることが、美咲には痛いほど伝わってきました。[PAUSE]しかし美咲は、この一週間で見てきた常連客たちの顔を思い浮かべました。杖をついて毎日通う田中さん、赤ちゃんを連れてくる若い母親、無口だけれど必ず顔を出す中年の男性。この銭湯がなくなれば、彼らの日課そのものが失われてしまう。美咲は思い切って、自分の貯金を取り崩し、新しいボイラーへの交換に踏み切ることを母に提案しました。[PAUSE]清子さんは、「そんな大金、娘に出させるわけにはいかない」と強く反対しましたが、美咲は「これは、私がこの三週間で学んだことへの恩返しだから」と譲りませんでした。押し問答の末、清子さんはようやく折れ、美咲の申し出を受け入れることにしました。工事の間、銭湯は一週間の臨時休業を余儀なくされましたが、常連客たちは口々に「待ってるから、ゆっくりやって」と温かい言葉をかけてくれました。休業中、美咲は毎日工事の様子を見に通い、慣れない専門用語に戸惑いながらも、業者とのやり取りや進捗の確認を一手に引き受けました。工事が完了した再開初日、田中さんをはじめとする常連客たちが次々と詰めかけ、「新しい湯船は気持ちいいねえ」と口々に喜びの声を上げました。[PAUSE]美咲が番台に座り続けるうちに、常連客たちも彼女に少しずつ心を開いていきました。ある日、いつも無口な男性客が、珍しく美咲に話しかけてきました。「俺は妻を亡くしてから、この銭湯だけが唯一の楽しみなんだ。清子さんも、あんたも、ここに座っていてくれるだけで、こっちは救われるんだよ」。美咲は、その言葉に深く胸を打たれました。[PAUSE]番台の手帳には、名前や好みだけでなく、声をかけると喜ぶ話題や、そっとしておいた方がよい日まで少しずつ増えていきました。美咲はそれを顧客名簿ではなく、母が長い歳月をかけて交わしてきた会話の地図なのだと思うようになりました。設備を守るだけでは、この場所は残らない。湯上がりの短い言葉を受け止める人がいてこそ、銭湯は町の居場所になるのだと分かったのです。手帳を開くたび、母の声が行間から聞こえるようでした。その声は、美咲が迷うたびに進む方角を静かに教えてくれました。[PAUSE]三週間後、清子さんはようやく体力を取り戻し、久しぶりに番台に戻ってきました。美咲は横に座り、清子さんが常連客たちと再会する様子を見守りました。「清子さん、待ってたよ」「元気になってよかった」。次々とかけられる温かい言葉に、清子さんは涙ぐみながら、深々と頭を下げていました。[PAUSE]帰りの荷造りをしながら、美咲はこの三週間の出来事を振り返り、まさか自分がこんなにも銭湯の仕事に心を動かされるとは思ってもみなかったと、一人静かに驚いていました。その夜、美咲は東京へ戻る支度をしながら、清子さんに切り出しました。「お母さん、私、月に一度でいいから、また帰ってきて番台に座らせてもらえないかな。すごく、大切な時間だったから」。清子さんは驚きながらも、嬉しそうに頷きました。それから美咲は、月に一度、実家に帰っては番台に座る生活を続けるようになりました。[PAUSE]月に一度の帰省が始まってから一年ほど経った頃、美咲は東京の職場で大きな昇進の話を持ちかけられました。海外支社への異動を伴う昇進で、これを受ければ、これまでのように月に一度実家に帰ることも難しくなります。美咲は、これまで積み上げてきたキャリアと、銭湯での大切な時間との間で、深く思い悩むことになりました。[PAUSE]美咲は上司に少し考えさせてほしいと伝え、次の帰省の際、清子さんにこの話を打ち明けました。清子さんは黙って話を聞いたあと、「あなたの人生よ。私のことは気にしなくていい。銭湯は、いつか閉めることになっても仕方ないんだから」と、寂しさを押し殺すように言いました。その言葉とは裏腹に、清子さんの目には隠しきれない切なさがにじんでいました。[PAUSE]その晩、美咲は眠れないまま、番台に一人座ってみました。閉店後の静まり返った浴室に、かつて聞いた常連客たちの声がよみがえってきます。「清子さんも、あんたも、ここに座っていてくれるだけで、こっちは救われるんだよ」。あの無口な男性客の言葉が、繰り返し頭の中に響きました。美咲は、この場所が自分にとってもかけがえのないものになっていることに、改めて気づかされました。[PAUSE]眠れないまま迎えた朝、美咲は洗面所の鏡に映る自分の顔を見つめ、これまでの数年間で自分がどれほど変わったかを実感しました。東京で働いていた頃には見えなかった、人と人との細やかなつながりの尊さに、この銭湯を通じて気づかされていたのです。翌朝、美咲は昇進の話を丁重に断ることに決めました。上司には、家庭の事情があると正直に伝え、代わりに国内での別の役職に就かせてもらえないか相談しました。上司は少し驚いた様子でしたが、美咲の真剣な表情を見て、「そこまで大切に思える場所があるのは、うらやましいことだよ」と言い、希望を聞き入れてくれました。[PAUSE]決断を伝える前夜、美咲は東京の静かな自分の部屋で一人、これまで築いてきたキャリアの重みと、銭湯で過ごした短い日々の温かさを、天秤にかけるように何度も考え直していました。特に親しくしていた先輩からは「せっかくここまで積み上げてきたのに」と心配され、他の同僚たちからも「もったいない」と惜しまれるだろうことも分かっていましたが、番台に座って感じたあの充足感に勝るものはないという確信だけは、揺らぐことがありませんでした。美咲がその決断を清子さんに伝えると、清子さんは驚きながらも、「無理はしないでほしい」と繰り返しました。美咲は首を横に振り、「無理をしているんじゃないの。ここが、私の大切な場所になったから、選んだだけ」と答えました。清子さんは、それ以上何も言わず、ただ静かに美咲の手を握りしめました。[PAUSE]それから美咲は、以前よりも頻繁に実家に帰るようになり、清子さんの体調が思わしくない日には、数日間泊まり込んで番台に座ることも増えていきました。常連客たちも、美咲が定期的に顔を出すことを当たり前のように受け止め、時には清子さんよりも先に、美咲に世間話を持ちかける客も出てくるようになりました。[PAUSE]数年後、清子さんが体力的に銭湯を続けるのが難しくなったとき、美咲は東京での仕事に区切りをつけ、正式に実家に戻って銭湯を継ぐことを決意しました。あの三週間で覚えた常連客たちの顔と名前は、すでに美咲の中でしっかりと根を張っていました。正式に番台を引き継ぐ日、清子さんは長年愛用してきた古い座布団を美咲に手渡しました。座布団の裏地には何度も繕われた跡があり、長い年月を物語っていました。「これに座って、初めてお客さんの顔をちゃんと見られるようになったの」と、清子さんは懐かしそうに目を細めました。清子さんは、番台を美咲に譲る日、静かにこう言いました。「この仕事は、体を洗う手伝いをするだけじゃない。人の暮らしに、ほんの少し寄り添う仕事なんだよ」。[PAUSE]美咲が正式に銭湯を継いでから二年ほど経った頃、思いがけない知らせが届きました。町の再開発計画により、銭湯のある一帯が数年以内に区画整理の対象になるかもしれないというのです。美咲は役所からの説明会に足を運び、詳しい事情を確認しました。計画が実行されれば、銭湯の建物も立ち退きの対象になる可能性があるとのことでした。[PAUSE]美咲はこの話を聞いて、目の前が真っ暗になるような気持ちを味わいました。せっかく母から受け継ぎ、常連客たちとの絆を築いてきたこの場所が、行政の計画一つで失われてしまうかもしれない。美咲は居ても立ってもいられず、同じように影響を受ける近隣の商店主たちと連絡を取り合い、対策を考える集まりを開くことにしました。[PAUSE]集まりには、長年この商店街で店を構えてきた人々が次々と参加しました。美咲は、銭湯が単なる入浴施設ではなく、高齢者たちの見守りの場、地域の交流の場としての役割を果たしていることを、これまでの経験をもとに説明しました。参加者たちは、それぞれの店が持つ地域での役割について語り合い、行政に対して再開発計画の見直しを求める要望書をまとめることになりました。[PAUSE]要望書の作成にあたり、美咲は自分の手帳に書き留めてきた常連客たちの記録を活用することにしました。誰が何年通っているか、銭湯がどんな役割を果たしてきたか、具体的な数字と共に文書にまとめていきました。田中さんをはじめとする常連客たちも、自ら役所に足を運び、直接自分たちの思いを伝えてくれました。[PAUSE]話し合いの中で、行政の担当者は当初、地域の意見をあまり重視しない姿勢を見せていましたが、美咲たちが粘り強く何度も足を運び、実際の利用状況や高齢者たちの声を届け続けるうちに、次第にその態度も軟化していきました。ある担当者は、「これほど地域に根ざした場所だとは、正直、想像していませんでした」と率直に語り、住民側の主張に理解を示すようになりました。数ヶ月にわたる話し合いの末、行政側は計画を全面的に見直し、銭湯を含む一角については、再開発の対象から除外するという決定を下しました。説明会の場で、この結果を聞いた美咲は、思わずその場に座り込みそうになるほどの安堵を覚えました。田中さんは美咲の肩を叩き、「あんたが頑張ってくれたおかげだ」と、目を潤ませながら言いました。[PAUSE]要望書をまとめる過程で、美咲は普段あまり関わりのなかった隣の惣菜屋の店主や、向かいのクリーニング店の若い店主とも、初めてじっくり言葉を交わす機会を得ました。それぞれが抱える悩みは違っていても、地域の人々を支えたいという思いは共通していることに気づき、美咲はこの商店街全体が、目に見えない形で支え合っていたのだと実感しました。この出来事をきっかけに、美咲は商店街の若手経営者たちとのつながりを深め、月に一度の情報交換会を自ら呼びかけて始めるなど、地域全体で高齢者を支える緩やかなネットワークづくりにも関わるようになりました。銭湯という一つの場所を守るために始めた行動が、思いがけず町全体を巻き込む大きな動きへとつながっていったのです。美咲は今も、あの手帳を大切に手元に置いています。新しい客が来るたびに、名前と特徴を書き足しながら、清子さんが四十年かけて築いてきたものを、少しずつ自分の手で育て直しているのです。白い湯気の立ちのぼる銭湯の向こうには、今日もたくさんの顔なじみが、いつも変わらぬ笑顔で美咲を迎えてくれます。[PAUSE]銭湯が存続することになったあの年の冬、清子さんは静かに息を引き取りました。最期の時、清子さんは病室から美咲の手を握り、「あなたが継いでくれて、本当によかった」と、かすれた声で伝えました。葬儀には、田中さんをはじめとする常連客たちが数多く参列し、清子さんとの思い出を涙ながらに語り合いました。[PAUSE]母を失った悲しみの中でも、美咲は毎日欠かさず番台に座り続けました。悲しみに沈んでいる暇はないというよりも、番台に座り、常連客たちと言葉を交わすことこそが、美咲にとって一番の慰めになっていたのです。ある日、いつもの無口な男性客が、珍しく長く話し込んでいきました。「清子さんも、きっとこの湯気の向こうから見てるよ」。その一言に、美咲は静かに涙をこぼしました。[PAUSE]銭湯を一人で切り盛りする日々の中で、美咲は自分の体力の限界も感じるようになっていました。朝早くから夜遅くまでボイラーの管理から番台、清掃までをすべて一人でこなすのは、想像以上に重労働でした。ある晩、美咲は疲れ果てて番台に突っ伏したまま眠り込んでしまい、翌朝、早くに来た常連の女性客に心配されて起こされるということもありました。「一人で全部背負い込まなくていいのよ」。その女性客の言葉が、美咲の胸に深く残りました。[PAUSE]母の死から半年ほど経ったある日、美咲のもとに、遠方に住む親戚から思いがけない相談が寄せられました。親戚の息子である健太という青年が、就職先が決まらず将来に悩んでいるので、しばらく銭湯の手伝いをさせてもらえないかというのです。美咲は、かつての自分自身と重ねながら、快く健太を受け入れることにしました。[PAUSE]健太は色白で物静かな青年で、人前に立つと緊張のあまり言葉が詰まってしまう性格でしたが、面接ではうまく自分を表現できず、いくつもの会社から立て続けに不採用の通知を受け取っていました。両親からも「もっと積極的にならないと」と言われ続け、すっかり自信を失っていました。美咲は、あえて仕事の細かい指示を多く出さず、まずは常連客たちとの何気ない会話に慣れてもらうことから始めました。最初はぎこちなかった健太も、田中さんに冗談を返されて思わず笑ってしまうなど、少しずつ肩の力が抜けていく様子が見て取れました。健太は最初こそ慣れない仕事に戸惑いながらも、美咲の丁寧な指導のもと、少しずつ番台の仕事を覚えていきました。美咲は、かつて清子さんが自分にしてくれたように、焦らず一人一人の常連客の顔と名前を覚えるよう、根気強く健太に教えました。あの手帳は、こうして三代目の記録として、新しいページが加えられていくことになったのです。[PAUSE]ある日、健太が思い切って美咲にこう打ち明けました。「正直、最初はただの腰かけのつもりでした。でも、常連さんたちが名前を覚えて声をかけてくれるようになって、自分が誰かに必要とされてるって実感が持てたんです」。美咲は、その言葉を聞きながら、かつて自分自身が抱いた思いと重なる部分に、深くうなずきました。健太は半年ほど手伝ううちに、それまでの弱気な表情が嘘のように明るくなり、この仕事に本気で向き合いたいという気持ちを固め、正式に銭湯で働かせてほしいと美咲に申し出ました。美咲はその申し出を喜んで受け入れ、いずれは健太にも、この場所の大切さを引き継いでいってほしいと願うようになりました。清子さんから美咲へ、そして美咲から健太へと、番台に込められた思いは、静かに、しかし確かに受け継がれていったのです。[PAUSE]急な、思いがけない出来事がきっかけで、誰かの大切な場所を引き継ぐことになる。そんなとき、大きな不安や戸惑いの中にも、これまで気づかなかった大切な尊さが隠れていることがあるのかもしれません。今夜の長いお話は、ここまでです。どうか安心して、今夜もゆっくりとお休みください。良い夢を。ゆっくり、おやすみなさい。</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2109,17 +2109,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>차례상 위에서 사라진 송편 한 개</t>
+          <t>닫힌 구둣방 문 앞에 놓인 국화 한 송이</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>안녕하세요. 9월 23일 수요일 아침입니다.[PAUSE]어젯밤 제사상에 올려 둔 송편이, 오늘 아침 보니 하나가 줄어 있었습니다. 가족들에게 물어봐도 아무도 손댄 적이 없다고 합니다. 창문은 닫혀 있었고, 고양이가 닿을 높이도 아니었습니다. 조금 이상하다 싶으면서도, '올해도 잘 전해졌나 보다' 하는 생각에 마음이 따뜻해졌습니다. 어머니가 살아 계실 때, 이맘때면 부엌에서 솔잎 찌는 냄새가 온 집 안에 퍼지곤 했던 기억이 납니다.[PAUSE]오늘 9월 23일은 추분입니다. 태양이 적도 위를 지나며 낮과 밤의 길이가 거의 같아지는 절기로, 예로부터 한 해 농사를 돌아보고 감사를 표하는 시기로 여겨져 왔습니다. 이 무렵이면 오곡백과가 무르익어, 옛사람들은 하늘에 감사하는 제를 올리기도 했다고 전해집니다.[PAUSE]추분을 지나면 이제부터 밤이 낮보다 조금씩 길어지기 시작합니다. 공기도 한층 맑아져서, 멀리 있는 산의 능선까지 또렷하게 보이는 날이 늘어날 것입니다. 마당의 감나무에도 주홍빛이 슬슬 돌기 시작하는 계절입니다.[PAUSE]오늘 성묘를 다녀오실 분들도 많을 것 같습니다. 서두르지 마시고, 소중한 분들과의 시간을 천천히 보내시길 바랍니다. 돌아오는 길에는 평소보다 조금 천천히 걸으며, 물들기 시작한 나뭇잎들을 눈에 담아 보시는 것도 좋겠습니다. 그럼 햇살 편지는 내일도 함께하겠습니다.</t>
+          <t>안녕하세요. 9월 23일 수요일 아침입니다.[PAUSE]동네에서 마흔 해 넘게 구두를 고쳐 온 영수 씨는 오늘만큼은 가게 문을 열지 않으려 했습니다. 아내가 세상을 떠난 뒤 처음 맞는 추분이라, 아침 일찍 산소에 다녀올 생각이었기 때문입니다. 그런데 셔터를 내린 구둣방 앞에 흰 국화 한 송이와 짧은 쪽지가 놓여 있었습니다. "아저씨가 고쳐 주신 신발 덕분에 첫 출근을 무사히 했습니다. 오늘은 편히 다녀오세요." 지난주, 닳은 면접 구두를 들고 왔던 청년이 남긴 인사였습니다. 영수 씨는 한참 쪽지를 바라보다 국화를 조심스레 가방에 넣었습니다. 오늘 아내에게 들려줄 이야기가 하나 더 생겼습니다.[PAUSE]오늘 9월 23일은 낮과 밤의 길이가 거의 같아지는 절기, 추분입니다. 추분을 지나면 밤이 조금씩 길어지고, 들판의 곡식과 과일은 한층 깊은 빛으로 익어 갑니다.[PAUSE]올해 추석은 이틀 뒤인 9월 25일입니다. 벌초나 성묘를 준비하신다면 아직 한낮 햇볕이 따가울 수 있으니 물을 챙기고, 무리하지 않는 것이 좋겠습니다. 멀리 이동하지 못하더라도 마음속으로 안부를 건네는 것만으로 충분한 날도 있습니다.[PAUSE]오늘은 영수 씨의 구둣방처럼 잠시 닫힌 문 앞에서도 따뜻한 마음 하나를 발견하는 하루가 되면 좋겠습니다. 여러분의 수요일 아침이 천천히, 평안하게 시작되길 바랍니다. 햇살 편지는 내일 다시 찾아오겠습니다.</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>아침,추분,성묘</t>
+          <t>아침,추분,추석</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2130,27 +2130,27 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
-          <t>추석 성묘 이야기</t>
+          <t>추분 아침 인사</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>추석 성묘 이야기 | 차례상 위에서 사라진 송편 한 개</t>
+          <t>추분 아침 인사 | 닫힌 구둣방 문 앞에 놓인 국화 한 송이</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>추석 차례상 위에서 사라진 송편 한 개를 둘러싼, 정겹고 훈훈한 수요일 아침 이야기입니다.</t>
+          <t>아내를 먼저 보낸 뒤 처음 맞는 추분 아침, 구둣방 앞에 놓인 국화 한 송이가 전해 준 작은 이야기입니다.</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>추석,성묘,아침인사,시니어콘텐츠,감성라디오</t>
+          <t>추분,추석,아침인사,시니어콘텐츠,감성라디오</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>#추석,#성묘,#아침인사,#시니어콘텐츠</t>
+          <t>#추분,#추석,#아침인사,#시니어콘텐츠</t>
         </is>
       </c>
     </row>
@@ -2177,12 +2177,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>옛이야기 인물 다섯 문제</t>
+          <t>한국과 일본 옛이야기 다섯 문제</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>안녕하세요. 점심시간 두뇌 퀴즈입니다. 오늘은 한국과 일본의 옛이야기에 등장하는 인물에 관한 문제 다섯 가지를 준비했습니다. 어릴 적 들었던 이야기를 떠올리며 함께 풀어 보시죠. 두 나라 모두, 오랜 세월 입에서 입으로 전해 내려온 소중한 이야기들입니다.[PAUSE]첫 번째 문제입니다. 제비 다리를 고쳐 주고 복을 받은 착한 동생의 이름은 무엇일까요?[PAUSE]정답은 '흥부'입니다. 욕심 많은 형 놀부와 대비되는 인물로, 제비가 물어다 준 박씨를 심어 큰 복을 받게 되는 이야기는 지금도 널리 사랑받고 있습니다. 형제간의 우애와 권선징악이라는 주제가 세대를 넘어 꾸준히 전해지는 이유이기도 합니다.[PAUSE]두 번째 문제입니다. 일본의 옛이야기에서, 할아버지가 산에서 주워 온 커다란 복숭아에서 태어난 아이는 누구일까요?[PAUSE]정답은 '모모타로'입니다. 개, 원숭이, 꿩을 데리고 도깨비를 물리치러 떠나는 이야기로, 일본에서는 어린이들이 가장 먼저 접하는 옛이야기 중 하나로 꼽힙니다.[PAUSE]세 번째 문제입니다. 계모와 언니들의 구박을 받다가, 원님과 혼인하게 되는 한국의 옛이야기 속 여인은 누구일까요?[PAUSE]정답은 '콩쥐'입니다. 콩쥐팥쥐 이야기 속에서, 착하고 성실한 콩쥐가 여러 시련을 이겨 내고 행복을 찾는 과정은 신데렐라 이야기와 비슷한 구조를 지녔다고도 이야기됩니다.[PAUSE]네 번째 문제입니다. 일본 옛이야기에서, 용궁에서 받아 온 상자를 열자 순식간에 노인이 되어 버린 어부의 이름은 무엇일까요?[PAUSE]정답은 '우라시마 타로'입니다. 거북이를 구해 준 보답으로 용궁에 초대받았지만, 절대 열지 말라던 상자를 열어 세월의 흐름을 한꺼번에 맞이하게 되는 이야기입니다.[PAUSE]마지막 문제입니다. 방망이를 두드리면 원하는 것이 나오는, 한국 옛이야기 속 신비한 도구를 손에 넣은 나무꾼과 관련된 이야기는 무엇일까요?[PAUSE]정답은 '도깨비 방망이'입니다. 정직한 나무꾼이 도깨비들의 방망이를 얻어 부자가 되지만, 이를 욕심으로 흉내 낸 이웃은 오히려 화를 입는다는 교훈적인 이야기로 전해집니다. 정직하게 살아가는 사람에게 복이 돌아온다는 메시지는 지금도 여러 이야기 속에서 되풀이되는 주제입니다.[PAUSE]다섯 문제 모두 풀어 보셨나요? 한국과 일본의 옛이야기에는 착함과 정직함이 결국 복으로 돌아온다는 공통된 가르침이 담겨 있는 듯합니다. 나라는 달라도, 오래도록 소중히 여겨 온 마음은 서로 닮아 있는 것 같습니다. 오늘은 어떤 이야기가 가장 기억에 남으셨나요? 손주나 자녀에게 오늘 배운 이야기를 들려주시는 것도 즐거운 시간이 될 것입니다. 그럼 내일 퀴즈에서 다시 뵙겠습니다.</t>
+          <t>안녕하세요. 점심시간 두뇌 퀴즈입니다. 오늘은 한국과 일본의 옛이야기에 등장인물과 신비한 물건에 관한 문제 다섯 가지를 준비했습니다. 어릴 적 들었던 이야기를 떠올리며 함께 풀어 보시죠. 두 나라 모두, 오랜 세월 입에서 입으로 전해 내려온 소중한 이야기들입니다.[PAUSE]첫 번째 문제입니다. 제비 다리를 고쳐 주고 복을 받은 착한 동생의 이름은 무엇일까요?[PAUSE]정답은 '흥부'입니다. 욕심 많은 형 놀부와 대비되는 인물로, 제비가 물어다 준 박씨를 심어 큰 복을 받게 되는 이야기는 지금도 널리 사랑받고 있습니다. 형제간의 우애와 권선징악이라는 주제가 세대를 넘어 꾸준히 전해지는 이유이기도 합니다.[PAUSE]두 번째 문제입니다. 일본의 옛이야기에서, 할아버지가 산에서 주워 온 커다란 복숭아에서 태어난 아이는 누구일까요?[PAUSE]정답은 '모모타로'입니다. 개, 원숭이, 꿩을 데리고 도깨비를 물리치러 떠나는 이야기로, 일본에서는 어린이들이 가장 먼저 접하는 옛이야기 중 하나로 꼽힙니다.[PAUSE]세 번째 문제입니다. 계모와 언니들의 구박을 받다가, 원님과 혼인하게 되는 한국의 옛이야기 속 여인은 누구일까요?[PAUSE]정답은 '콩쥐'입니다. 콩쥐팥쥐 이야기 속에서, 착하고 성실한 콩쥐가 여러 시련을 이겨 내고 행복을 찾는 과정은 신데렐라 이야기와 비슷한 구조를 지녔다고도 이야기됩니다.[PAUSE]네 번째 문제입니다. 일본 옛이야기에서, 용궁에서 받아 온 상자를 열자 순식간에 노인이 되어 버린 어부의 이름은 무엇일까요?[PAUSE]정답은 '우라시마 타로'입니다. 거북이를 구해 준 보답으로 용궁에 초대받았지만, 절대 열지 말라던 상자를 열어 세월의 흐름을 한꺼번에 맞이하게 되는 이야기입니다.[PAUSE]마지막 문제입니다. 방망이를 두드리면 원하는 것이 나오는, 한국 옛이야기 속 신비한 도구를 손에 넣은 나무꾼과 관련된 이야기는 무엇일까요?[PAUSE]정답은 '도깨비 방망이'입니다. 정직한 나무꾼이 도깨비들의 방망이를 얻어 부자가 되지만, 이를 욕심으로 흉내 낸 이웃은 오히려 화를 입는다는 교훈적인 이야기로 전해집니다. 정직하게 살아가는 사람에게 복이 돌아온다는 메시지는 지금도 여러 이야기 속에서 되풀이되는 주제입니다.[PAUSE]다섯 문제 모두 풀어 보셨나요? 한국과 일본의 옛이야기에는 착함과 정직함이 결국 복으로 돌아온다는 공통된 가르침이 담겨 있는 듯합니다. 나라는 달라도, 오래도록 소중히 여겨 온 마음은 서로 닮아 있는 것 같습니다. 오늘은 어떤 이야기가 가장 기억에 남으셨나요? 손주나 자녀에게 오늘 배운 이야기를 들려주시는 것도 즐거운 시간이 될 것입니다. 그럼 내일 퀴즈에서 다시 뵙겠습니다.</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2203,12 +2203,12 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>옛이야기 퀴즈 | 한일 옛이야기 인물 다섯 문제</t>
+          <t>옛이야기 퀴즈 | 한국과 일본 옛이야기 다섯 문제</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>한국과 일본에 전해 내려오는 옛이야기 속 인물들을 다루는 다섯 문제 두뇌 퀴즈입니다.</t>
+          <t>한국과 일본의 서로 다른 옛이야기 속 등장인물과 신비한 물건을 맞히는 다섯 문제 두뇌 퀴즈입니다.</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>빨간 우산 벤치 추억 | 오십 년 만에 풀린 태식 씨의 물음표 (실화 감성)</t>
+          <t>빨간 우산 벤치 추억 | 오십 년 만에 풀린 태식 씨의 물음표</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2285,12 +2285,12 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>빨간 우산 벤치 추억,옛사랑 이야기,실화 감성 스토리,시니어 콘텐츠,추억 라디오,어르신 이야기</t>
+          <t>빨간 우산 벤치 추억,옛 인연 이야기,감성 창작 스토리,시니어 콘텐츠,추억 라디오,어르신 이야기</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>#빨간우산,#벤치추억,#옛사랑이야기,#실화감성,#시니어라디오</t>
+          <t>#빨간우산,#벤치추억,#옛인연이야기,#감성스토리,#시니어라디오</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>화요일 오후 세 시, 화양극장 영사실 안에서 병철 씨는 벤허 두 번째 릴을 영사기에 걸고 있었습니다. 필름 오른쪽 위 모서리, 장면이 끝나기 팔 초 전에 나타나는 작은 점 두 개, 그 체인지 마크를 서른 해 가까이 놓친 적이 없었습니다.[PAUSE]체인지 마크가 화면 구석에 깜박이는 순간, 병철 씨는 곧바로 옆에 세워 둔 두 번째 영사기의 스타트 버튼을 눌렀습니다. 두 대의 영사기가 겹치는 이삼 초 사이, 객석에서는 아무도 눈치채지 못할 만큼 매끄럽게 화면이 이어졌습니다. 이 감각 하나를 익히는 데만도, 병철 씨는 신입 시절 꼬박 두 해를 보냈습니다.[PAUSE]안녕하세요.[PAUSE]이 늦은 시각까지 햇살 편지를 찾아 주셔서 고맙습니다.[PAUSE]하루를 마무리하며, 조용히 마음을 내려놓아 보세요.[PAUSE]병철 씨는 올해 예순넷, 이 작은 단관 극장의 영사실을 서른두 해째 지켜 온 사람입니다. 두 대의 영사기를 번갈아 돌리며 릴이 바뀌는 순간을 감쪽같이 이어 붙이는 일, 렌즈의 초점과 화면 비율을 필름 상태에 맞춰 미세하게 조정하는 일, 그리고 상영 도중 필름이 끊어졌을 때 객석에서 눈치채지 못하게 이 분 안에 스플라이서로 이어 붙이는 일까지, 모두 병철 씨의 손끝에서 나온 기술이었습니다.[PAUSE]필름이 낡아 화면이 지지직거리거나 색이 바랬을 때, 렌즈 조리개를 미세하게 조절해 관객이 눈치채지 못할 정도로만 화면을 보정하는 것도 병철 씨만의 요령이었습니다. 매표소 직원들조차 어떤 영화가 원래 상태가 좋고 나쁜지 모를 정도로, 병철 씨의 손을 거치면 낡은 필름도 제법 매끈하게 살아났습니다.[PAUSE]지난달, 극장 사장 강 사장님은 영사실 벽에 공고문 한 장을 붙였습니다. 이번 분기를 끝으로 필름 영사기를 완전히 철거하고, 극장을 디지털 상영관으로 전환한다는 내용이었습니다. 서른두 해 동안 병철 씨가 지켜 온 이 영사실에서, 필름을 거는 일은 이번 달이 마지막이 될 예정이었습니다.[PAUSE]공고문이 붙은 날, 매표소 직원 미영 씨가 조심스럽게 물었습니다. "아저씨, 이제 필름 영사기 다루는 사람 필요 없어지는 거예요?" 병철 씨는 옅게 웃으며 대답했습니다. "디지털은 버튼 하나만 누르면 되니까. 이제 이런 손재주는 필요 없어지는 거지." 후임을 따로 뽑을 계획도 없다는 것을, 병철 씨는 이미 알고 있었습니다.[PAUSE]병철 씨가 이 일을 처음 배운 것은 스물두 살, 서울의 한 개봉관 견습 영사기사로 들어갔을 때였습니다. 당시 선배 기사가 던져 준 필름 조각을 붙잡고 밤새 스플라이서 다루는 법을 익히던 기억이, 지금도 손끝에 고스란히 남아 있었습니다. 그 뒤로 이 화양극장에 자리를 잡기까지, 병철 씨는 전국의 크고 작은 극장 영사실을 두루 거쳤습니다.[PAUSE]그 소식을 들은 뒤로도 병철 씨는 평소와 다름없이 매일 오후 세 시면 영사실에 올라와 그날 상영할 필름을 점검했습니다. 릴을 손으로 돌려 가며 필름 표면에 흠집은 없는지, 이음새가 뜯어진 곳은 없는지 확인하는 일은, 이제 와 새삼 배운 습관이 아니라 몸에 밴 하루의 시작이었습니다.[PAUSE]화양극장에는 수요일 낮마다 빠짐없이 오는 단골손님이 있었습니다. 정순 할머니, 올해 여든하나로, 이십 년 넘게 매주 수요일 두 시 회차를 지켜 온 분이었습니다. 병철 씨는 표를 받을 때마다 얼굴만 보고도 정순 할머니가 어느 줄, 몇 번째 자리에 앉을지 알 정도였습니다.[PAUSE]정순 할머니는 늘 상영 시작 이십 분 전에 도착해, 매표소 옆 자판기 커피를 한 잔 뽑아 들고 로비 의자에 앉아 있곤 했습니다. 병철 씨는 영사실로 올라가는 길에 종종 인사를 나누었고, 몇 해 전부터는 굳이 묻지 않아도 정순 할머니가 그날 매점에서 무엇을 살지 짐작할 수 있을 정도가 되었습니다.[PAUSE]그런데 언젠가부터 정순 할머니의 발걸음이 뜸해지더니, 두 달 가까이 극장에 모습을 보이지 않았습니다. 병철 씨는 그저 몸이 편찮으신가 보다 짐작만 할 뿐이었습니다. 그러던 어느 날 오후, 정순 할머니가 딸의 부축을 받으며 매표소 앞에 나타났습니다. 이전보다 훨씬 야윈 모습이었습니다. 병철 씨는 반가운 마음에 인사를 건넸지만, 정순 할머니는 힘겹게 손을 내저으며 오늘은 영화를 보러 온 것이 아니라고 말했습니다.[PAUSE]정순 할머니는 매표소 직원이 아니라 굳이 영사실 앞까지 딸의 부축을 받으며 걸어 올라와, 병철 씨를 찾았습니다. "병철 씨, 나 부탁이 하나 있어서 왔어요." 딸이 조심스럽게 사정을 대신 설명했습니다. 어머니가 위암 말기 판정을 받아 이제 남은 시간이 길지 않다는 것, 그리고 마지막으로 꼭 보고 싶은 영화가 있다는 것이었습니다.[PAUSE]정순 할머니가 말한 영화는 "미워도 다시 한번"이었습니다. "우리 영감이랑 결혼하고 얼마 안 됐을 때, 이 극장에서 같이 봤던 영화예요. 그이가 십 년 전에 먼저 갔는데, 죽기 전에 그 영화를 다시 한번 이 극장에서 보고 싶다고, 늘 노래처럼 말했었어요." 정순 할머니의 목소리는 낮았지만 또렷했습니다. "이제 저도 얼마 안 남았다고 하니, 그이한테 가서 대신 봤다고 말해 주고 싶어서요."[PAUSE]병철 씨는 곧바로 필름 보관고로 내려가 재고 목록을 확인했습니다. 혹시나 하는 마음에 비슷한 시기에 나온 다른 필름 상자 몇 개를 함께 꺼내 살펴보았지만, 그 영화만은 유일하게 한 벌만 남아 있었고, 다른 지방 극장이나 필름 보관소에도 남은 프린트가 없다는 것을 전화로 확인했습니다. 그 영화의 필름은 극장 창고 맨 안쪽, 십 년 넘게 한 번도 꺼내 쓰지 않은 릴 하나가 전부였습니다. 상자를 열자마자 시큼한 식초 냄새가 훅 끼쳐 올라왔습니다. 필름이 삭아 갈 때 나는 냄새, 이른바 초산 증후군이었습니다.[PAUSE]릴을 조심스럽게 풀어 손끝으로 필름을 훑어 보니, 표면 곳곳이 누렇게 뒤틀려 있었고, 스프로킷 구멍 몇 군데는 이미 잘게 갈라진 상태였습니다. 예전에 급하게 이어 붙였던 접합 부위 두 곳은 접착제가 삭아 손끝이 살짝 스치기만 해도 떨어질 듯 위태로웠습니다. 이대로 영사기에 걸었다가는, 렌즈 앞 뜨거운 게이트를 지나며 그대로 타 버리거나 찢어질 위험이 컸습니다. 병철 씨는 릴을 다시 상자에 담으며, 이 필름을 무사히 돌리려면 단순한 점검을 넘어선 손질이 필요하다는 것을 직감했습니다.[PAUSE]병철 씨는 이 사정을 강 사장님에게 그대로 전했습니다. 강 사장님은 단호하게 고개를 저었습니다. "안 돼요. 이번 달 안에 영사기 인수자한테 넘겨야 하는데, 그 필름 걸다가 게이트라도 상하면 어쩔 겁니까. 그리고 그 영화, 디지털 파일도 없잖아요." 실제로 그 영화는 복원 작업이 이루어지지 않아, 디지털 상영본 자체가 존재하지 않는 작품이었습니다.[PAUSE]강 사장님의 말도 틀리지 않았습니다. 영사기는 이미 지방의 한 필름 영사기 전시관으로 넘어가기로 계약이 끝난 상태였고, 인수 검수 날짜까지 정해져 있었습니다. 게이트 부품이 손상되면 인수 자체가 무산될 수도 있었습니다. 병철 씨는 그 자리에서 물러서지 않고 다시 한번 청했습니다. "제가 근무 시간 끝나고 따로 손봐 보겠습니다. 극장 이름으로 상영하는 게 아니라, 제 개인적인 부탁이라고 생각해 주십시오." 강 사장님은 한참 말이 없다가, 짧게 한숨을 내쉬었습니다. "정 그러시다면, 대신 문제가 생겨도 극장 책임은 아닙니다."[PAUSE]병철 씨는 그 조건을 그대로 받아들였습니다. 인수자 측에는 아직 알리지 않은 채, 정해진 검수일 전까지 조용히 마무리 짓기로 했습니다. 무거운 마음을 안고 병철 씨는 다시 영사실로 돌아왔습니다.[PAUSE]그날 밤, 병철 씨는 퇴근하지 않고 홀로 영사실에 남았습니다. 낡은 필름 릴을 다시 꺼내 형광등 아래 펼쳐 놓고, 한 프레임씩 손으로 짚어 가며 살펴보았습니다. 서른두 해 동안 수천 개의 필름을 만져 온 손이었지만, 이토록 삭은 필름을 되살려 본 적은 없었습니다.[PAUSE]병철 씨는 정순 할머니의 얼굴을 떠올렸습니다. 십 년 전 남편을 먼저 보내고도 매주 수요일마다 이 극장을 찾아온 사람, 이제는 살아 있는 날이 얼마 남지 않은 사람의 마지막 부탁이었습니다. 실패하면 필름은 완전히 망가지고, 상영 당일 손님들 앞에서 극장이 망신을 당할 수도 있는 일이었습니다. 병철 씨는 그래도 해 보기로, 조용히 마음을 굳혔습니다.[PAUSE]다음 날부터 병철 씨는 정규 근무를 마친 뒤, 퇴근 시간 이후에 혼자 남아 필름 복구 작업에 매달렸습니다. 삭은 접착 부위를 조심스럽게 떼어 내고, 필름 전용 세척액으로 눌어붙은 이물질을 하나하나 닦아 냈습니다. 갈라진 스프로킷 구멍 주변은 얇은 필름 테이프로 보강해, 영사기 톱니에 걸릴 때 더 이상 찢어지지 않도록 손을 보았습니다.[PAUSE]필름이 뒤틀리는 것을 막기 위해, 병철 씨는 영사실 습도를 일정하게 맞추려고 낡은 가습기까지 창고에서 꺼내 왔습니다. 너무 건조하면 필름이 바스러지고, 너무 습하면 곰팡이가 슬기 쉬웠습니다. 이런 세심한 조건을 맞추는 일은, 매뉴얼 어디에도 적혀 있지 않은, 오직 병철 씨의 경험으로만 아는 요령이었습니다.[PAUSE]가장 까다로운 것은 접합 부위였습니다. 병철 씨는 오래된 필름 스플라이서를 꺼내, 삭은 부분을 정확히 몇 밀리미터 잘라 내고 새로 이어 붙이는 작업을 시작했습니다. 그런데 첫 번째 접합은 접착액이 채 마르기도 전에 손끝이 스치면서 다시 떨어져 나가고 말았습니다. 필름 한 조각이 허무하게 못 쓰게 되는 순간이었습니다.[PAUSE]병철 씨는 잠시 손을 멈추고 숨을 골랐습니다. 여기서 또 실패하면 남은 필름 길이로는 접합을 다시 시도할 여유조차 없었습니다. 그는 접착액의 양을 훨씬 적게 조절하고, 누르는 시간을 평소보다 두 배로 늘려 가며 두 번째 접합을 시도했습니다. 이번에는 접합 부위가 단단하게 붙었습니다.[PAUSE]그렇게 사흘 밤을 꼬박 매달려, 병철 씨는 릴 전체의 접합 부위 여섯 곳을 모두 손보았습니다. 작업을 마친 뒤에도 안심할 수 없었던 병철 씨는, 영사기가 아닌 손 감기용 리와인더에 필름을 걸어 몇 번이고 천천히 돌려 보며 걸리는 곳은 없는지, 접합 부위가 버티는지 확인하고 또 확인했습니다.[PAUSE]셋째 날 새벽, 병철 씨는 문득 이 모든 일이 부질없는 고집일지도 모른다는 생각에 잠시 손을 놓았습니다. 실패하면 결국 정순 할머니에게 못 보여 드리게 될 뿐 아니라, 하나 남은 필름마저 영영 잃게 되는 것이었습니다. 그러나 병철 씨는 이내 다시 스플라이서를 집어 들었습니다. 여기서 멈추면, 시도조차 하지 않은 것을 훗날 더 크게 후회할 것 같았습니다.[PAUSE]상영 예정일 전날 밤, 병철 씨는 마지막으로 영사기에 필름을 걸고 초저속으로 시험 가동을 해 보았습니다. 필름은 게이트를 무사히 통과했지만, 후반부 한 접합 지점에서 아주 미세하게 걸리는 느낌이 손끝에 전해졌습니다. 완벽하지 않다는 것을 알면서도, 병철 씨에게는 더 이상 손볼 시간이 남아 있지 않았습니다.[PAUSE]드디어 상영 날, 정순 할머니는 딸의 부축을 받으며 평소 앉던 그 자리에 앉았습니다. 소문을 들은 동네 노인정 어르신들 몇 분과, 정순 할머니의 오랜 이웃들도 함께 표를 끊어 객석 여기저기에 자리를 잡았습니다. 작은 극장 안이 오랜만에 손님들로 제법 채워졌습니다.[PAUSE]강 사장님은 걱정스러운 얼굴로 객석 뒤편에 서서 상영을 지켜보았습니다. 병철 씨는 영사실 창을 통해 정순 할머니의 뒷모습을 확인한 뒤, 조용히 영사기의 스위치를 올렸습니다.[PAUSE]영화가 시작되고 첫 번째 릴이 무사히 돌아가는 동안, 병철 씨는 필름이 지나가는 소리 하나하나에 온 신경을 곤두세우고 있었습니다. 평소라면 신경 쓰지 않았을 사소한 마찰음까지도, 오늘만큼은 병철 씨의 귀에 유독 크게 울렸습니다. 손끝은 언제든 영사기 손잡이를 붙잡을 수 있도록 릴 옆에서 떨어지지 않았습니다.[PAUSE]문제는 후반부, 병철 씨가 미리 걱정했던 바로 그 접합 지점에서 터졌습니다. 화면이 순간적으로 파르르 떨리더니, 필름이 게이트 안에서 살짝 걸리는 느낌이 손잡이를 통해 전해졌습니다. 조금만 늦으면 필름이 그대로 찢어지거나 뜨거운 램프 열에 눌어붙을 수 있는 순간이었습니다.[PAUSE]병철 씨는 반사적으로 영사기 손잡이를 붙잡아 속도를 아주 미세하게 늦추고, 다른 손으로는 필름이 걸린 부위를 살짝 밀어 텐션을 풀어 주었습니다. 객석에서는 화면이 잠깐 흔들린 것 정도로만 보였을, 몇 초 안 되는 그 순간에, 병철 씨의 등줄기에는 식은땀이 흘러내리고 있었습니다.[PAUSE]다행히 필름은 걸린 부위를 무사히 빠져나갔고, 화면은 다시 안정을 되찾았습니다. 병철 씨는 그제야 참았던 숨을 길게 내쉬었습니다. 손바닥은 땀으로 흠뻑 젖어 있었고, 심장은 여전히 세차게 뛰고 있었습니다. 남은 상영 시간 동안 병철 씨는 단 한순간도 영사기 앞을 떠나지 않고, 필름이 돌아가는 모든 소리에 귀를 기울였습니다.[PAUSE]영화가 끝나고 마지막 자막이 다 지나갈 때까지, 필름은 더 이상 아무 문제 없이 끝까지 돌아갔습니다. 객석에 불이 켜지자, 정순 할머니는 손수건으로 눈가를 오래도록 닦아 내고 있었습니다. 딸이 손을 잡아 드리며 무슨 말인가 나누는 모습이, 영사실 창 너머로 병철 씨에게도 보였습니다.[PAUSE]정순 할머니는 딸의 부축을 받으며 극장을 나서기 전, 일부러 매표소 옆 계단을 통해 영사실 앞까지 다시 걸음을 옮겼습니다. 좁은 계단을 한 칸씩 딸의 부축을 받으며 오르는 그 모습이, 병철 씨에게는 유난히 오래 눈에 남았습니다. 병철 씨가 문을 열고 나오자, 정순 할머니는 두 손으로 병철 씨의 손을 꼭 잡았습니다. "고마워요. 우리 영감이랑 여기 앉아서 그 영화 보던 그날로 돌아간 것 같았어요."[PAUSE]병철 씨는 별다른 대답을 하지 못하고 그저 고개를 숙였습니다. 정순 할머니는 그런 병철 씨를 향해 조용히 웃으며 한마디를 더 남겼습니다. "이 나이에 이런 호사를 누릴 줄은 몰랐어요. 병철 씨 덕분에 여한이 없어졌어요." 그 말을 끝으로 정순 할머니는 딸의 팔에 기대어 천천히 극장 문을 나섰습니다.[PAUSE]그로부터 세 달 뒤, 정순 할머니의 딸이 극장으로 작은 화분 하나를 들고 찾아왔습니다. 딸은 병철 씨에게 어머니가 두 주 전 편안하게 눈을 감으셨다는 소식을 전했습니다. "돌아가시기 전까지, 그날 영화 본 이야기를 몇 번이고 하셨어요. 병철 씨한테 꼭 고맙다는 말을 다시 전해 달라고 하셨습니다." 병철 씨는 화분을 영사실 창가에 조용히 올려 두었습니다.[PAUSE]딸은 돌아가기 전, 병철 씨에게 사진 한 장을 보여 주었습니다. 그날 상영이 끝난 뒤 로비에서 찍은 것으로, 정순 할머니가 오랜만에 환하게 웃고 있는 모습이었습니다. "엄마가 그렇게 웃으신 거, 정말 오랜만이었어요." 병철 씨는 그 사진을 한참 동안 들여다보다가, 조심스럽게 휴대전화로 옮겨 담았습니다.[PAUSE]그 뒤로도 극장의 마지막 한 달은 빠르게 흘러갔습니다. 병철 씨는 여느 때처럼 매일 오후 세 시면 영사실에 올라와 그날의 필름을 점검했고, 밤이 되면 마지막 회차의 필름을 되감아 정리했습니다. 다만 이제는 그 하루하루가 정말 얼마 남지 않았다는 것을, 병철 씨 스스로도 또렷이 느끼고 있었습니다.[PAUSE]폐관 소식이 지역 신문에 짧게 실리자, 오랫동안 발길이 뜸했던 옛 단골들이 하나둘 다시 극장을 찾아왔습니다. 개중에는 정순 할머니의 사연을 전해 듣고 일부러 찾아와, 병철 씨에게 자신도 옛날에 좋아했던 영화를 마지막으로 한 번만 틀어 줄 수 있는지 조심스럽게 물어보는 손님도 있었습니다. 병철 씨는 남은 필름 재고가 허락하는 한, 그런 부탁들을 하나씩 들어주었습니다.[PAUSE]극장의 마지막 상영일 아침, 강 사장님은 병철 씨를 조용히 불러 지난 일에 대해 짧게 사과했습니다. "그때는 미안했어요. 필름 상태를 직접 보지도 않고 무조건 안 된다고만 했으니." 병철 씨는 괜찮다는 뜻으로 고개를 끄덕이며, 정순 할머니가 두고 간 화분을 가리켰습니다. "저것 때문에라도, 그날 걸어 보길 잘했다는 생각이 듭니다."[PAUSE]마지막 상영이 끝난 그날 저녁, 병철 씨는 영사실에 마지막으로 홀로 남아 영사기 전원을 내렸습니다. 서른두 해 동안 수만 번 오르내렸던 계단, 필름 냄새와 기름 냄새가 배어든 이 좁은 방을, 병철 씨는 천천히 눈에 담았습니다. 창밖으로 보이는 극장 앞 골목 풍경도, 이제는 마지막으로 보는 것이라 생각하니 유독 낯설게 느껴졌습니다.[PAUSE]다음 날, 필름 영사기 전시관에서 나온 사람들이 영사기를 분해해 트럭에 싣기 시작했습니다. 병철 씨는 직접 나사를 하나하나 풀어내며, 인수자들에게 렌즈 관리법과 게이트 청소 요령을 하나씩 일러 주었습니다. 이 영사기가 폐기되지 않고 전시관에 보존되어, 앞으로도 다른 사람들이 필름 영사의 원리를 볼 수 있게 된다는 것이, 병철 씨에게는 작은 위안이었습니다.[PAUSE]매표소 미영 씨는 마지막까지 남아 영사기가 실려 나가는 모습을 지켜보다가, 병철 씨에게 다가와 조용히 말을 건넸습니다. "아저씨, 그동안 고생 많으셨어요. 이제 뭐 하실 거예요?" 병철 씨는 잠시 생각하다가 대답했습니다. "당분간은 좀 쉬어야지. 그리고 가끔은 저 전시관에 놀러 가서, 저 녀석 잘 지내는지 들여다볼 생각이야."[PAUSE]영사기가 실려 나가는 모습을 지켜보며, 병철 씨는 지난 서른두 해를 돌이켜 보았습니다. 이 기술을 물려받을 사람도, 뒤를 이을 사람도 이제는 없다는 사실이 못내 허전했지만, 병철 씨는 그것을 아쉬움으로만 남겨 두지 않기로 했습니다. 트럭이 골목을 빠져나가는 뒷모습을 보며, 병철 씨는 오히려 홀가분한 마음이 조금씩 차오르는 것을 느꼈습니다.[PAUSE]병철 씨는 정순 할머니가 두고 간 화분을 품에 안고 극장 계단을 내려오며 생각했습니다. 서른두 해 동안 지켜 온 것은 결국 필름을 돌리는 기술 그 자체가 아니라, 그 기술을 통해 누군가의 마지막 소원을 들어줄 수 있었던 순간들이었다는 것을 말입니다.[PAUSE]만약 그날 밤 필름을 고치지 않고 강 사장님의 말대로 영사기만 지켰더라면, 영사기는 흠집 하나 없이 전시관에 넘어갔을지 모릅니다. 검수 당일에도 아무런 문제 없이 인수는 무사히 끝났고, 강 사장님은 그제야 병철 씨의 손끝이 얼마나 정확했는지 새삼 알게 되었다며 고개를 절레절레 흔들었습니다. 하지만 병철 씨는 그보다, 낡은 필름을 다시 살려 한 사람의 마지막 부탁을 지켜 낸 그 밤을 훨씬 더 소중하게 여기고 있었습니다.[PAUSE]장비를 아끼는 것도, 정해진 규정을 따르는 것도 물론 중요한 일입니다. 그러나 때로는 그 모든 것보다, 눈앞에 있는 한 사람의 간절한 마지막 부탁에 손을 내미는 일이 더 값진 선택일 수 있다는 것을, 병철 씨는 그 겨울 서른두 해 만에 새삼 깨달았습니다. 누군가에게 물려줄 기술은 없었지만, 그 밤의 선택 하나만큼은 병철 씨 스스로에게 오래도록 남을 유산이 되었습니다.[PAUSE]오늘 밤의 이 이야기는 여기서 마치겠습니다. 낡고 삭은 것이라 해도, 누군가에게는 평생을 담아 온 소중한 기억일 수 있습니다. 그 기억을 지켜 내려는 작은 용기가, 때로는 가장 큰 기술보다 더 오래 남는다는 것을 기억해 주시면 좋겠습니다. 편안한 마음으로, 부디 오늘 밤도 푹 주무시길 바랍니다. 좋은 꿈 꾸시고, 오늘 밤도 참으로 따뜻하고 평온한 밤 보내시길 바랍니다. 안녕히 주무세요, 여러분.</t>
+          <t>화요일 오후 세 시, 화양극장 영사실 안에서 병철 씨는 벤허 두 번째 릴을 영사기에 걸고 있었습니다. 필름 오른쪽 위 모서리, 장면이 끝나기 팔 초 전에 나타나는 작은 점 두 개, 그 체인지 마크를 서른 해 가까이 놓친 적이 없었습니다.[PAUSE]체인지 마크가 화면 구석에 깜박이는 순간, 병철 씨는 곧바로 옆에 세워 둔 두 번째 영사기의 스타트 버튼을 눌렀습니다. 두 대의 영사기가 겹치는 이삼 초 사이, 객석에서는 아무도 눈치채지 못할 만큼 매끄럽게 화면이 이어졌습니다. 이 감각 하나를 익히는 데만도, 병철 씨는 신입 시절 꼬박 두 해를 보냈습니다.[PAUSE]안녕하세요.[PAUSE]이 늦은 시각까지 햇살 편지를 찾아 주셔서 고맙습니다.[PAUSE]하루를 마무리하며, 조용히 마음을 내려놓아 보세요.[PAUSE]병철 씨는 올해 예순넷, 이 작은 단관 극장의 영사실을 서른두 해째 지켜 온 사람입니다. 두 대의 영사기를 번갈아 돌리며 릴이 바뀌는 순간을 감쪽같이 이어 붙이는 일, 렌즈의 초점과 화면 비율을 필름 상태에 맞춰 미세하게 조정하는 일, 그리고 상영 도중 필름이 끊어졌을 때 객석에서 눈치채지 못하게 이 분 안에 스플라이서로 이어 붙이는 일까지, 모두 병철 씨의 손끝에서 나온 기술이었습니다.[PAUSE]필름이 낡아 화면이 지지직거리거나 색이 바랬을 때, 렌즈 조리개를 미세하게 조절해 관객이 눈치채지 못할 정도로만 화면을 보정하는 것도 병철 씨만의 요령이었습니다. 매표소 직원들조차 어떤 영화가 원래 상태가 좋고 나쁜지 모를 정도로, 병철 씨의 손을 거치면 낡은 필름도 제법 매끈하게 살아났습니다.[PAUSE]지난달, 극장 사장 강 사장님은 영사실 벽에 공고문 한 장을 붙였습니다. 이번 분기를 끝으로 필름 영사기를 완전히 철거하고, 극장을 디지털 상영관으로 전환한다는 내용이었습니다. 서른두 해 동안 병철 씨가 지켜 온 이 영사실에서, 필름을 거는 일은 이번 달이 마지막이 될 예정이었습니다.[PAUSE]공고문이 붙은 날, 매표소 직원 미영 씨가 조심스럽게 물었습니다. "아저씨, 이제 필름 영사기 다루는 사람 필요 없어지는 거예요?" 병철 씨는 옅게 웃으며 대답했습니다. "디지털은 버튼 하나만 누르면 되니까. 이제 이런 손재주는 필요 없어지는 거지." 후임을 따로 뽑을 계획도 없다는 것을, 병철 씨는 이미 알고 있었습니다.[PAUSE]병철 씨가 이 일을 처음 배운 것은 스물두 살, 서울의 한 개봉관 견습 영사기사로 들어갔을 때였습니다. 당시 선배 기사가 던져 준 필름 조각을 붙잡고 밤새 스플라이서 다루는 법을 익히던 기억이, 지금도 손끝에 고스란히 남아 있었습니다. 그 뒤로 이 화양극장에 자리를 잡기까지, 병철 씨는 전국의 크고 작은 극장 영사실을 두루 거쳤습니다.[PAUSE]그 소식을 들은 뒤로도 병철 씨는 평소와 다름없이 매일 오후 세 시면 영사실에 올라와 그날 상영할 필름을 점검했습니다. 릴을 손으로 돌려 가며 필름 표면에 흠집은 없는지, 이음새가 뜯어진 곳은 없는지 확인하는 일은, 이제 와 새삼 배운 습관이 아니라 몸에 밴 하루의 시작이었습니다.[PAUSE]화양극장에는 수요일 낮마다 빠짐없이 오는 단골손님이 있었습니다. 정순 할머니, 올해 여든하나로, 이십 년 넘게 매주 수요일 두 시 회차를 지켜 온 분이었습니다. 병철 씨는 표를 받을 때마다 얼굴만 보고도 정순 할머니가 어느 줄, 몇 번째 자리에 앉을지 알 정도였습니다.[PAUSE]정순 할머니는 늘 상영 시작 이십 분 전에 도착해, 매표소 옆 자판기 커피를 한 잔 뽑아 들고 로비 의자에 앉아 있곤 했습니다. 병철 씨는 영사실로 올라가는 길에 종종 인사를 나누었고, 몇 해 전부터는 굳이 묻지 않아도 정순 할머니가 그날 매점에서 무엇을 살지 짐작할 수 있을 정도가 되었습니다.[PAUSE]그런데 언젠가부터 정순 할머니의 발걸음이 뜸해지더니, 두 달 가까이 극장에 모습을 보이지 않았습니다. 병철 씨는 그저 몸이 편찮으신가 보다 짐작만 할 뿐이었습니다. 그러던 어느 날 오후, 정순 할머니가 딸의 부축을 받으며 매표소 앞에 나타났습니다. 이전보다 훨씬 야윈 모습이었습니다. 병철 씨는 반가운 마음에 인사를 건넸지만, 정순 할머니는 힘겹게 손을 내저으며 오늘은 영화를 보러 온 것이 아니라고 말했습니다.[PAUSE]정순 할머니는 매표소 직원이 아니라 굳이 영사실 앞까지 딸의 부축을 받으며 걸어 올라와, 병철 씨를 찾았습니다. "병철 씨, 나 부탁이 하나 있어서 왔어요." 딸이 조심스럽게 사정을 대신 설명했습니다. 어머니가 위암 말기 판정을 받아 이제 남은 시간이 길지 않다는 것, 그리고 마지막으로 꼭 보고 싶은 영화가 있다는 것이었습니다.[PAUSE]정순 할머니가 말한 영화는 "그해 겨울의 편지"이었습니다. "우리 영감이랑 결혼하고 얼마 안 됐을 때, 이 극장에서 같이 봤던 영화예요. 그이가 십 년 전에 먼저 갔는데, 죽기 전에 그 영화를 다시 한번 이 극장에서 보고 싶다고, 늘 노래처럼 말했었어요." 정순 할머니의 목소리는 낮았지만 또렷했습니다. "이제 저도 얼마 안 남았다고 하니, 그이한테 가서 대신 봤다고 말해 주고 싶어서요."[PAUSE]병철 씨는 곧바로 필름 보관고로 내려가 재고 목록을 확인했습니다. 혹시나 하는 마음에 비슷한 시기에 나온 다른 필름 상자 몇 개를 함께 꺼내 살펴보았지만, 그 영화만은 유일하게 한 벌만 남아 있었고, 다른 지방 극장이나 필름 보관소에도 남은 프린트가 없다는 것을 전화로 확인했습니다. 그 영화의 필름은 극장 창고 맨 안쪽, 십 년 넘게 한 번도 꺼내 쓰지 않은 릴 하나가 전부였습니다. 상자를 열자마자 시큼한 식초 냄새가 훅 끼쳐 올라왔습니다. 필름이 삭아 갈 때 나는 냄새, 이른바 초산 증후군이었습니다.[PAUSE]릴을 조심스럽게 풀어 손끝으로 필름을 훑어 보니, 표면 곳곳이 누렇게 뒤틀려 있었고, 스프로킷 구멍 몇 군데는 이미 잘게 갈라진 상태였습니다. 예전에 급하게 이어 붙였던 접합 부위 두 곳은 접착제가 삭아 손끝이 살짝 스치기만 해도 떨어질 듯 위태로웠습니다. 이대로 영사기에 걸었다가는, 렌즈 앞 뜨거운 게이트를 지나며 그대로 타 버리거나 찢어질 위험이 컸습니다. 병철 씨는 릴을 다시 상자에 담으며, 이 필름을 무사히 돌리려면 단순한 점검을 넘어선 손질이 필요하다는 것을 직감했습니다.[PAUSE]병철 씨는 이 사정을 강 사장님에게 그대로 전했습니다. 강 사장님은 단호하게 고개를 저었습니다. "안 돼요. 이번 달 안에 영사기 인수자한테 넘겨야 하는데, 그 필름 걸다가 게이트라도 상하면 어쩔 겁니까. 그리고 그 영화, 디지털 파일도 없잖아요." 오래전 이 극장에서 잠깐 상영한 독립영화라 정식 디지털 상영본을 구할 수 없는 작품이었습니다.[PAUSE]강 사장님의 말도 틀리지 않았습니다. 영사기는 이미 지방의 한 필름 영사기 전시관으로 넘어가기로 계약이 끝난 상태였고, 인수 검수 날짜까지 정해져 있었습니다. 게이트 부품이 손상되면 인수 자체가 무산될 수도 있었습니다. 병철 씨는 그 자리에서 물러서지 않고 다시 한번 청했습니다. "제가 근무 시간 끝나고 따로 손봐 보겠습니다. 극장 이름으로 상영하는 게 아니라, 제 개인적인 부탁이라고 생각해 주십시오." 강 사장님은 한참 말이 없다가, 짧게 한숨을 내쉬었습니다. "정 그러시다면, 대신 문제가 생겨도 극장 책임은 아닙니다."[PAUSE]병철 씨는 그 조건을 그대로 받아들였습니다. 인수자 측에는 아직 알리지 않은 채, 정해진 검수일 전까지 조용히 마무리 짓기로 했습니다. 무거운 마음을 안고 병철 씨는 다시 영사실로 돌아왔습니다.[PAUSE]그날 밤, 병철 씨는 퇴근하지 않고 홀로 영사실에 남았습니다. 낡은 필름 릴을 다시 꺼내 형광등 아래 펼쳐 놓고, 한 프레임씩 손으로 짚어 가며 살펴보았습니다. 서른두 해 동안 수천 개의 필름을 만져 온 손이었지만, 이토록 삭은 필름을 되살려 본 적은 없었습니다.[PAUSE]병철 씨는 정순 할머니의 얼굴을 떠올렸습니다. 십 년 전 남편을 먼저 보내고도 매주 수요일마다 이 극장을 찾아온 사람, 이제는 살아 있는 날이 얼마 남지 않은 사람의 마지막 부탁이었습니다. 실패하면 필름은 완전히 망가지고, 상영 당일 손님들 앞에서 극장이 망신을 당할 수도 있는 일이었습니다. 병철 씨는 그래도 해 보기로, 조용히 마음을 굳혔습니다.[PAUSE]다음 날부터 병철 씨는 정규 근무를 마친 뒤, 퇴근 시간 이후에 혼자 남아 필름 복구 작업에 매달렸습니다. 삭은 접착 부위를 조심스럽게 떼어 내고, 필름 전용 세척액으로 눌어붙은 이물질을 하나하나 닦아 냈습니다. 갈라진 스프로킷 구멍 주변은 얇은 필름 테이프로 보강해, 영사기 톱니에 걸릴 때 더 이상 찢어지지 않도록 손을 보았습니다.[PAUSE]필름이 뒤틀리는 것을 막기 위해, 병철 씨는 영사실 습도를 일정하게 맞추려고 낡은 가습기까지 창고에서 꺼내 왔습니다. 너무 건조하면 필름이 바스러지고, 너무 습하면 곰팡이가 슬기 쉬웠습니다. 이런 세심한 조건을 맞추는 일은, 매뉴얼 어디에도 적혀 있지 않은, 오직 병철 씨의 경험으로만 아는 요령이었습니다.[PAUSE]가장 까다로운 것은 접합 부위였습니다. 병철 씨는 오래된 필름 스플라이서를 꺼내, 삭은 부분을 정확히 몇 밀리미터 잘라 내고 새로 이어 붙이는 작업을 시작했습니다. 그런데 첫 번째 접합은 접착액이 채 마르기도 전에 손끝이 스치면서 다시 떨어져 나가고 말았습니다. 필름 한 조각이 허무하게 못 쓰게 되는 순간이었습니다.[PAUSE]병철 씨는 잠시 손을 멈추고 숨을 골랐습니다. 여기서 또 실패하면 남은 필름 길이로는 접합을 다시 시도할 여유조차 없었습니다. 그는 접착액의 양을 훨씬 적게 조절하고, 누르는 시간을 평소보다 두 배로 늘려 가며 두 번째 접합을 시도했습니다. 이번에는 접합 부위가 단단하게 붙었습니다.[PAUSE]그렇게 사흘 밤을 꼬박 매달려, 병철 씨는 릴 전체의 접합 부위 여섯 곳을 모두 손보았습니다. 작업을 마친 뒤에도 안심할 수 없었던 병철 씨는, 영사기가 아닌 손 감기용 리와인더에 필름을 걸어 몇 번이고 천천히 돌려 보며 걸리는 곳은 없는지, 접합 부위가 버티는지 확인하고 또 확인했습니다.[PAUSE]셋째 날 새벽, 병철 씨는 문득 이 모든 일이 부질없는 고집일지도 모른다는 생각에 잠시 손을 놓았습니다. 실패하면 결국 정순 할머니에게 못 보여 드리게 될 뿐 아니라, 하나 남은 필름마저 영영 잃게 되는 것이었습니다. 그러나 병철 씨는 이내 다시 스플라이서를 집어 들었습니다. 여기서 멈추면, 시도조차 하지 않은 것을 훗날 더 크게 후회할 것 같았습니다.[PAUSE]상영 예정일 전날 밤, 병철 씨는 마지막으로 영사기에 필름을 걸고 초저속으로 시험 가동을 해 보았습니다. 필름은 게이트를 무사히 통과했지만, 후반부 한 접합 지점에서 아주 미세하게 걸리는 느낌이 손끝에 전해졌습니다. 완벽하지 않다는 것을 알면서도, 병철 씨에게는 더 이상 손볼 시간이 남아 있지 않았습니다.[PAUSE]드디어 상영 날, 정순 할머니는 딸의 부축을 받으며 평소 앉던 그 자리에 앉았습니다. 소문을 들은 동네 노인정 어르신들 몇 분과, 정순 할머니의 오랜 이웃들도 함께 표를 끊어 객석 여기저기에 자리를 잡았습니다. 작은 극장 안이 오랜만에 손님들로 제법 채워졌습니다.[PAUSE]강 사장님은 걱정스러운 얼굴로 객석 뒤편에 서서 상영을 지켜보았습니다. 병철 씨는 영사실 창을 통해 정순 할머니의 뒷모습을 확인한 뒤, 조용히 영사기의 스위치를 올렸습니다.[PAUSE]영화가 시작되고 첫 번째 릴이 무사히 돌아가는 동안, 병철 씨는 필름이 지나가는 소리 하나하나에 온 신경을 곤두세우고 있었습니다. 평소라면 신경 쓰지 않았을 사소한 마찰음까지도, 오늘만큼은 병철 씨의 귀에 유독 크게 울렸습니다. 손끝은 언제든 영사기 손잡이를 붙잡을 수 있도록 릴 옆에서 떨어지지 않았습니다.[PAUSE]문제는 후반부, 병철 씨가 미리 걱정했던 바로 그 접합 지점에서 터졌습니다. 화면이 순간적으로 파르르 떨리더니, 필름이 게이트 안에서 살짝 걸리는 느낌이 손잡이를 통해 전해졌습니다. 조금만 늦으면 필름이 그대로 찢어지거나 뜨거운 램프 열에 눌어붙을 수 있는 순간이었습니다.[PAUSE]병철 씨는 반사적으로 영사기 손잡이를 붙잡아 속도를 아주 미세하게 늦추고, 다른 손으로는 필름이 걸린 부위를 살짝 밀어 텐션을 풀어 주었습니다. 객석에서는 화면이 잠깐 흔들린 것 정도로만 보였을, 몇 초 안 되는 그 순간에, 병철 씨의 등줄기에는 식은땀이 흘러내리고 있었습니다.[PAUSE]다행히 필름은 걸린 부위를 무사히 빠져나갔고, 화면은 다시 안정을 되찾았습니다. 병철 씨는 그제야 참았던 숨을 길게 내쉬었습니다. 손바닥은 땀으로 흠뻑 젖어 있었고, 심장은 여전히 세차게 뛰고 있었습니다. 남은 상영 시간 동안 병철 씨는 단 한순간도 영사기 앞을 떠나지 않고, 필름이 돌아가는 모든 소리에 귀를 기울였습니다.[PAUSE]영화가 끝나고 마지막 자막이 다 지나갈 때까지, 필름은 더 이상 아무 문제 없이 끝까지 돌아갔습니다. 객석에 불이 켜지자, 정순 할머니는 손수건으로 눈가를 오래도록 닦아 내고 있었습니다. 딸이 손을 잡아 드리며 무슨 말인가 나누는 모습이, 영사실 창 너머로 병철 씨에게도 보였습니다.[PAUSE]정순 할머니는 딸의 부축을 받으며 극장을 나서기 전, 일부러 매표소 옆 계단을 통해 영사실 앞까지 다시 걸음을 옮겼습니다. 좁은 계단을 한 칸씩 딸의 부축을 받으며 오르는 그 모습이, 병철 씨에게는 유난히 오래 눈에 남았습니다. 병철 씨가 문을 열고 나오자, 정순 할머니는 두 손으로 병철 씨의 손을 꼭 잡았습니다. "고마워요. 우리 영감이랑 여기 앉아서 그 영화 보던 그날로 돌아간 것 같았어요."[PAUSE]병철 씨는 별다른 대답을 하지 못하고 그저 고개를 숙였습니다. 정순 할머니는 그런 병철 씨를 향해 조용히 웃으며 한마디를 더 남겼습니다. "이 나이에 이런 호사를 누릴 줄은 몰랐어요. 병철 씨 덕분에 여한이 없어졌어요." 그 말을 끝으로 정순 할머니는 딸의 팔에 기대어 천천히 극장 문을 나섰습니다.[PAUSE]그로부터 세 달 뒤, 정순 할머니의 딸이 극장으로 작은 화분 하나를 들고 찾아왔습니다. 딸은 병철 씨에게 어머니가 두 주 전 편안하게 눈을 감으셨다는 소식을 전했습니다. "돌아가시기 전까지, 그날 영화 본 이야기를 몇 번이고 하셨어요. 병철 씨한테 꼭 고맙다는 말을 다시 전해 달라고 하셨습니다." 병철 씨는 화분을 영사실 창가에 조용히 올려 두었습니다.[PAUSE]딸은 돌아가기 전, 병철 씨에게 사진 한 장을 보여 주었습니다. 그날 상영이 끝난 뒤 로비에서 찍은 것으로, 정순 할머니가 오랜만에 환하게 웃고 있는 모습이었습니다. "엄마가 그렇게 웃으신 거, 정말 오랜만이었어요." 병철 씨는 그 사진을 한참 동안 들여다보다가, 조심스럽게 휴대전화로 옮겨 담았습니다.[PAUSE]그 뒤로도 극장의 마지막 한 달은 빠르게 흘러갔습니다. 병철 씨는 여느 때처럼 매일 오후 세 시면 영사실에 올라와 그날의 필름을 점검했고, 밤이 되면 마지막 회차의 필름을 되감아 정리했습니다. 다만 이제는 그 하루하루가 정말 얼마 남지 않았다는 것을, 병철 씨 스스로도 또렷이 느끼고 있었습니다.[PAUSE]폐관 소식이 지역 신문에 짧게 실리자, 오랫동안 발길이 뜸했던 옛 단골들이 하나둘 다시 극장을 찾아왔습니다. 개중에는 정순 할머니의 사연을 전해 듣고 일부러 찾아와, 병철 씨에게 자신도 옛날에 좋아했던 영화를 마지막으로 한 번만 틀어 줄 수 있는지 조심스럽게 물어보는 손님도 있었습니다. 병철 씨는 남은 필름 재고가 허락하는 한, 그런 부탁들을 하나씩 들어주었습니다.[PAUSE]극장의 마지막 상영일 아침, 강 사장님은 병철 씨를 조용히 불러 지난 일에 대해 짧게 사과했습니다. "그때는 미안했어요. 필름 상태를 직접 보지도 않고 무조건 안 된다고만 했으니." 병철 씨는 괜찮다는 뜻으로 고개를 끄덕이며, 정순 할머니가 두고 간 화분을 가리켰습니다. "저것 때문에라도, 그날 걸어 보길 잘했다는 생각이 듭니다."[PAUSE]마지막 상영이 끝난 그날 저녁, 병철 씨는 영사실에 마지막으로 홀로 남아 영사기 전원을 내렸습니다. 서른두 해 동안 수만 번 오르내렸던 계단, 필름 냄새와 기름 냄새가 배어든 이 좁은 방을, 병철 씨는 천천히 눈에 담았습니다. 창밖으로 보이는 극장 앞 골목 풍경도, 이제는 마지막으로 보는 것이라 생각하니 유독 낯설게 느껴졌습니다.[PAUSE]다음 날, 필름 영사기 전시관에서 나온 사람들이 영사기를 분해해 트럭에 싣기 시작했습니다. 병철 씨는 직접 나사를 하나하나 풀어내며, 인수자들에게 렌즈 관리법과 게이트 청소 요령을 하나씩 일러 주었습니다. 이 영사기가 폐기되지 않고 전시관에 보존되어, 앞으로도 다른 사람들이 필름 영사의 원리를 볼 수 있게 된다는 것이, 병철 씨에게는 작은 위안이었습니다.[PAUSE]매표소 미영 씨는 마지막까지 남아 영사기가 실려 나가는 모습을 지켜보다가, 병철 씨에게 다가와 조용히 말을 건넸습니다. "아저씨, 그동안 고생 많으셨어요. 이제 뭐 하실 거예요?" 병철 씨는 잠시 생각하다가 대답했습니다. "당분간은 좀 쉬어야지. 그리고 가끔은 저 전시관에 놀러 가서, 저 녀석 잘 지내는지 들여다볼 생각이야."[PAUSE]영사기가 실려 나가는 모습을 지켜보며, 병철 씨는 지난 서른두 해를 돌이켜 보았습니다. 이 기술을 물려받을 사람도, 뒤를 이을 사람도 이제는 없다는 사실이 못내 허전했지만, 병철 씨는 그것을 아쉬움으로만 남겨 두지 않기로 했습니다. 트럭이 골목을 빠져나가는 뒷모습을 보며, 병철 씨는 오히려 홀가분한 마음이 조금씩 차오르는 것을 느꼈습니다.[PAUSE]병철 씨는 정순 할머니가 두고 간 화분을 품에 안고 극장 계단을 내려오며 생각했습니다. 서른두 해 동안 지켜 온 것은 결국 필름을 돌리는 기술 그 자체가 아니라, 그 기술을 통해 누군가의 마지막 소원을 들어줄 수 있었던 순간들이었다는 것을 말입니다.[PAUSE]만약 그날 밤 필름을 고치지 않고 강 사장님의 말대로 영사기만 지켰더라면, 영사기는 흠집 하나 없이 전시관에 넘어갔을지 모릅니다. 검수 당일에도 아무런 문제 없이 인수는 무사히 끝났고, 강 사장님은 그제야 병철 씨의 손끝이 얼마나 정확했는지 새삼 알게 되었다며 고개를 절레절레 흔들었습니다. 하지만 병철 씨는 그보다, 낡은 필름을 다시 살려 한 사람의 마지막 부탁을 지켜 낸 그 밤을 훨씬 더 소중하게 여기고 있었습니다.[PAUSE]장비를 아끼는 것도, 정해진 규정을 따르는 것도 물론 중요한 일입니다. 그러나 때로는 그 모든 것보다, 눈앞에 있는 한 사람의 간절한 마지막 부탁에 손을 내미는 일이 더 값진 선택일 수 있다는 것을, 병철 씨는 그 겨울 서른두 해 만에 새삼 깨달았습니다. 누군가에게 물려줄 기술은 없었지만, 그 밤의 선택 하나만큼은 병철 씨 스스로에게 오래도록 남을 유산이 되었습니다.[PAUSE]오늘 밤의 이 이야기는 여기서 마치겠습니다. 낡고 삭은 것이라 해도, 누군가에게는 평생을 담아 온 소중한 기억일 수 있습니다. 그 기억을 지켜 내려는 작은 용기가, 때로는 가장 큰 기술보다 더 오래 남는다는 것을 기억해 주시면 좋겠습니다. 편안한 마음으로, 부디 오늘 밤도 푹 주무시길 바랍니다. 좋은 꿈 꾸시고, 오늘 밤도 참으로 따뜻하고 평온한 밤 보내시길 바랍니다. 안녕히 주무세요, 여러분.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -5276,7 +5276,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>桃から生まれた男の子の名前は？</t>
+          <t>桃から生まれ、鬼退治へ向かった主人公は？</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -5306,7 +5306,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>犬・猿・雉を家来にして鬼退治に向かう物語です。</t>
+          <t>犬・猿・雉にきびだんごを分けて仲間にします。</t>
         </is>
       </c>
     </row>
@@ -5323,37 +5323,37 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>天女の羽衣を隠した木こりの韓国の物語名は？</t>
+          <t>「フンブとノルブ」でフンブが助けた生き物は？</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ソンニョと木こり</t>
+          <t>つばめ</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>コンジとパッチ</t>
+          <t>うさぎ</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>フンブとノルブ</t>
+          <t>亀</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>トッケビの話</t>
+          <t>鶴</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>ソンニョと木こり</t>
+          <t>つばめ</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>地域によって結末が異なる伝承が残っています。</t>
+          <t>元気になったつばめが瓢箪の種を運びます。</t>
         </is>
       </c>
     </row>
@@ -5370,37 +5370,37 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>川上から流れてきて桃太郎が生まれたものは？</t>
+          <t>竹の中から現れ、月へ帰る主人公は？</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>瓜</t>
+          <t>かぐや姫</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>桃</t>
+          <t>乙姫</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>西瓜</t>
+          <t>鶴女房</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>栗</t>
+          <t>織姫</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>桃</t>
+          <t>かぐや姫</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>「おばあさんは川へ洗濯に」の場面で登場します。</t>
+          <t>「竹取物語」は日本最古の物語文学とされています。</t>
         </is>
       </c>
     </row>
@@ -5417,37 +5417,37 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>「フンブとノルブ」でフンブが助けた生き物は？</t>
+          <t>「コンジとパッチ」でコンジを助ける生き物の一つは？</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>つばめ</t>
+          <t>牛</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>うさぎ</t>
+          <t>狐</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>亀</t>
+          <t>鶴</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>鶴</t>
+          <t>虎</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>つばめ</t>
+          <t>牛</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>足を折ったつばめを助けたことで幸運を授かります。</t>
+          <t>伝承では牛やひきがえるなどが仕事を助けます。</t>
         </is>
       </c>
     </row>
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>浦島太郎が竜宮城から持ち帰った箱の名前は？</t>
+          <t>浦島太郎が持ち帰った箱の名前は？</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -5494,7 +5494,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>開けると煙が立ちのぼり一気に年をとる結末です。</t>
+          <t>開けると白い煙が立ちのぼる結末です。</t>
         </is>
       </c>
     </row>
@@ -7843,10 +7843,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>663</v>
+        <v>675</v>
       </c>
       <c r="F6" t="n">
-        <v>131.4</v>
+        <v>133.7</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -7881,10 +7881,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="F7" t="n">
-        <v>139.6</v>
+        <v>139.4</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -7919,10 +7919,10 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1239</v>
+        <v>1240</v>
       </c>
       <c r="F8" t="n">
-        <v>245.4</v>
+        <v>245.6</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -8029,14 +8029,14 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>차례상 위에서 사라진 송편 한 개</t>
+          <t>닫힌 구둣방 문 앞에 놓인 국화 한 송이</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>646</v>
+        <v>661</v>
       </c>
       <c r="F11" t="n">
-        <v>127.4</v>
+        <v>130.3</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -8071,10 +8071,10 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1213</v>
+        <v>1220</v>
       </c>
       <c r="F12" t="n">
-        <v>240.3</v>
+        <v>241.7</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -8105,14 +8105,14 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>옛이야기 인물 다섯 문제</t>
+          <t>한국과 일본 옛이야기 다섯 문제</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1230</v>
+        <v>1235</v>
       </c>
       <c r="F13" t="n">
-        <v>243.6</v>
+        <v>244.6</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -8869,10 +8869,10 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>9224</v>
+        <v>9214</v>
       </c>
       <c r="F33" t="n">
-        <v>1814</v>
+        <v>1812</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -8907,10 +8907,10 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>8544</v>
+        <v>8553</v>
       </c>
       <c r="F34" t="n">
-        <v>1680</v>
+        <v>1681.7</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -8945,10 +8945,10 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>9034</v>
+        <v>9031</v>
       </c>
       <c r="F35" t="n">
-        <v>1779.6</v>
+        <v>1779</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -9287,10 +9287,10 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>914</v>
+        <v>1755</v>
       </c>
       <c r="F44" t="n">
-        <v>180.3</v>
+        <v>346.4</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -9325,10 +9325,10 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>959</v>
+        <v>2113</v>
       </c>
       <c r="F45" t="n">
-        <v>189.1</v>
+        <v>416.3</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -9990,10 +9990,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G6" t="n">
         <v>100</v>
@@ -10201,14 +10201,14 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>차례상 위에서 사라진 송편 한 개</t>
+          <t>닫힌 구둣방 문 앞에 놓인 국화 한 송이</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F11" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G11" t="n">
         <v>100</v>
@@ -10248,10 +10248,10 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="F12" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="G12" t="n">
         <v>100</v>
@@ -10287,7 +10287,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>옛이야기 인물 다섯 문제</t>
+          <t>한국과 일본 옛이야기 다섯 문제</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -11151,10 +11151,10 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F33" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G33" t="n">
         <v>100</v>
@@ -11194,10 +11194,10 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F34" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G34" t="n">
         <v>100</v>
@@ -11624,10 +11624,10 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="F44" t="n">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="G44" t="n">
         <v>100</v>
@@ -11667,10 +11667,10 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>17</v>
+        <v>50</v>
       </c>
       <c r="F45" t="n">
-        <v>17</v>
+        <v>50</v>
       </c>
       <c r="G45" t="n">
         <v>100</v>

</xml_diff>